<commit_message>
ahl delegacije + statistika
</commit_message>
<xml_diff>
--- a/data/ICEHLdelegacije.xlsx
+++ b/data/ICEHLdelegacije.xlsx
@@ -16,7 +16,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="2075" uniqueCount="318">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="2076" uniqueCount="318">
   <si>
     <t>PiragicTr</t>
   </si>
@@ -675,7 +675,7 @@
     <t>Tiroler Wasserkraft Arena;SeewaldEl;SmetanaLa;MartinFl;RieckenSi</t>
   </si>
   <si>
-    <t>Sparkasse Arena Bozen;BernekerTh;NikolicKr;PuffWo;RigoniDa</t>
+    <t>Sparkasse Arena Bozen;BernekerTh;SchauerJa;PuffWo;RigoniDa</t>
   </si>
   <si>
     <t>Gabor Ocskay Eisarena;HronskyTo;PiragicTr;DurmisOt;HribarMa</t>
@@ -786,7 +786,7 @@
     <t>Hala Tivoli;GroznikBo;NagyAt;HribarMa;PuffWo</t>
   </si>
   <si>
-    <t>Eishalle Asiago;RezekGr;SchauerJa;HribarMa;PardatscherUl</t>
+    <t>Eishalle Asiago;GroznikBo;RezekGr;HribarMa;PardatscherUl</t>
   </si>
   <si>
     <t>Tiroler Wasserkraft Arena;NikolicKr;OfnerCh;BedynekSe;MartinFl</t>
@@ -831,7 +831,7 @@
     <t>Eisarena Salzburg;HronskyTo;SternatCh;JedlickaPe;SeewaldJe</t>
   </si>
   <si>
-    <t>Tiroler Wasserkraft Arena;NikolicKr;NikolicMa;MartinFl;SparerDa</t>
+    <t>Tiroler Wasserkraft Arena;NikolicMa;NikolicKr;MartinFl;SparerDa</t>
   </si>
   <si>
     <t>Eishalle Bruneck;BernekerTh;HuberAn;MartinFl;PardatscherUl</t>
@@ -3109,7 +3109,7 @@
         <v>96</v>
       </c>
       <c r="AI14" t="s">
-        <v>76</v>
+        <v>97</v>
       </c>
       <c r="AJ14" t="s">
         <v>96</v>
@@ -4195,8 +4195,11 @@
       <c r="D28" t="s">
         <v>77</v>
       </c>
+      <c r="F28" t="s">
+        <v>76</v>
+      </c>
     </row>
-    <row r="29" ht="15" customHeight="1" spans="1:4" x14ac:dyDescent="0.25">
+    <row r="29" ht="15" customHeight="1" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A29" t="s">
         <v>101</v>
       </c>
@@ -5956,7 +5959,7 @@
         <v>1</v>
       </c>
       <c r="AE13" t="s">
-        <v>34</v>
+        <v>24</v>
       </c>
       <c r="AF13" t="s">
         <v>0</v>
@@ -6301,7 +6304,7 @@
         <v>5</v>
       </c>
       <c r="AE16" t="s">
-        <v>23</v>
+        <v>5</v>
       </c>
       <c r="AF16" t="s">
         <v>34</v>
@@ -6346,7 +6349,7 @@
         <v>18</v>
       </c>
       <c r="BA16" t="s">
-        <v>34</v>
+        <v>6</v>
       </c>
     </row>
     <row r="17" ht="15" customHeight="1" spans="1:53" x14ac:dyDescent="0.25">
@@ -6405,7 +6408,7 @@
         <v>36</v>
       </c>
       <c r="AE17" t="s">
-        <v>24</v>
+        <v>23</v>
       </c>
       <c r="AF17" t="s">
         <v>2</v>
@@ -6450,7 +6453,7 @@
         <v>3</v>
       </c>
       <c r="BA17" t="s">
-        <v>6</v>
+        <v>34</v>
       </c>
     </row>
     <row r="18" ht="15" customHeight="1" spans="1:53" x14ac:dyDescent="0.25">

</xml_diff>

<commit_message>
ahl delegacije do 30.1
</commit_message>
<xml_diff>
--- a/data/ICEHLdelegacije.xlsx
+++ b/data/ICEHLdelegacije.xlsx
@@ -16,7 +16,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="2681" uniqueCount="398">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="2685" uniqueCount="399">
   <si>
     <t>SmetanaLa</t>
   </si>
@@ -300,6 +300,9 @@
     <t>2025-01-03</t>
   </si>
   <si>
+    <t>2025-01-24</t>
+  </si>
+  <si>
     <t>2024-10-23</t>
   </si>
   <si>
@@ -312,57 +315,57 @@
     <t>2025-01-10</t>
   </si>
   <si>
+    <t>zbrisano</t>
+  </si>
+  <si>
+    <t>2024-11-22</t>
+  </si>
+  <si>
+    <t>2024-12-01</t>
+  </si>
+  <si>
+    <t>2024-11-16</t>
+  </si>
+  <si>
+    <t>2024-12-04</t>
+  </si>
+  <si>
+    <t>2024-12-13</t>
+  </si>
+  <si>
+    <t>2024-12-30</t>
+  </si>
+  <si>
+    <t>2025-01-12</t>
+  </si>
+  <si>
+    <t>2024-11-30</t>
+  </si>
+  <si>
+    <t>2025-01-08</t>
+  </si>
+  <si>
+    <t>2024-11-23</t>
+  </si>
+  <si>
+    <t>2024-12-03</t>
+  </si>
+  <si>
+    <t>2024-12-15</t>
+  </si>
+  <si>
+    <t>2024-12-07</t>
+  </si>
+  <si>
+    <t>2025-01-17</t>
+  </si>
+  <si>
     <t>2025-01-26</t>
   </si>
   <si>
-    <t>2024-11-22</t>
-  </si>
-  <si>
-    <t>2024-12-01</t>
-  </si>
-  <si>
-    <t>2024-11-16</t>
-  </si>
-  <si>
-    <t>2024-12-04</t>
-  </si>
-  <si>
-    <t>2024-12-13</t>
-  </si>
-  <si>
-    <t>2024-12-30</t>
-  </si>
-  <si>
-    <t>2025-01-12</t>
-  </si>
-  <si>
-    <t>2024-11-30</t>
-  </si>
-  <si>
-    <t>2025-01-08</t>
-  </si>
-  <si>
-    <t>2024-11-23</t>
-  </si>
-  <si>
-    <t>2024-12-03</t>
-  </si>
-  <si>
-    <t>2024-12-15</t>
-  </si>
-  <si>
-    <t>2024-12-07</t>
-  </si>
-  <si>
-    <t>2025-01-17</t>
-  </si>
-  <si>
     <t>2024-12-14</t>
   </si>
   <si>
-    <t>2025-01-24</t>
-  </si>
-  <si>
     <t>2024-12-10</t>
   </si>
   <si>
@@ -723,7 +726,7 @@
     <t>Heidi Horten Arena Klagenfurt;FichtnerPa;SmetanaLa;BärnthalerCh;ZgoncGa</t>
   </si>
   <si>
-    <t>Tiroler Wasserkraft Arena;NikolicKr;NikolicMa;PardatscherUl;ZacherlPa</t>
+    <t>Tiroler Wasserkraft Arena;NikolicMa;NikolicKr;PardatscherUl;ZacherlPa</t>
   </si>
   <si>
     <t>Eishalle Feldkirch;BernekerTh;NikolicKr;MartinFl;SeewaldJe</t>
@@ -891,7 +894,7 @@
     <t>Tiroler Wasserkraft Arena;FichtnerPa;SiegelSt;MartinFl;PardatscherUl</t>
   </si>
   <si>
-    <t>Eishalle Feldkirch;OfnerCh;SternatCh;FleischmannLu;PardatscherUl</t>
+    <t>Eishalle Feldkirch;OfnerCh;SternatCh;PardatscherUl;SparerDa</t>
   </si>
   <si>
     <t>Stadthalle Villach;HronskyTo;ZrnicMi;DurmisOt;KoncDa</t>
@@ -1008,7 +1011,7 @@
     <t>Linz AG Eisarena;PiragicTr;SiegelSt;Gatol-schafranekMa;SeewaldJe</t>
   </si>
   <si>
-    <t>Linz AG Eisarena;Huber aAn;SmetanaLa;DurmisOt;NotheggerDa</t>
+    <t>Linz AG Eisarena;Huber aAn;SmetanaLa;NotheggerDa;WeissAl</t>
   </si>
   <si>
     <t>Stadthalle Villach;RezekGr;SmetanaLa;HribarMa;RieckenSi</t>
@@ -1119,13 +1122,13 @@
     <t>Hala Tivoli;GroznikBo;OfnerCh;MuzsikNo;VacziDa</t>
   </si>
   <si>
-    <t>Heidi Horten Arena Klagenfurt;HronskyTo;Huber aAn;BärnthalerCh;DurmisOt</t>
+    <t>Heidi Horten Arena Klagenfurt;HronskyTo;Huber aAn;BärnthalerCh;KoncDa</t>
   </si>
   <si>
     <t>Eishalle Asiago;SchauerJa;SternatCh;PardatscherUl;RigoniDa</t>
   </si>
   <si>
-    <t>Eishalle Asiago;OfnerCh;SternatCh;HribarMa;ZgoncGa</t>
+    <t>Eishalle Asiago;OfnerCh;SternatCh;JeramFi;ZgoncGa</t>
   </si>
   <si>
     <t>Tiroler Wasserkraft Arena;BernekerTh;OfnerCh;MartinFl;SeewaldJe</t>
@@ -2783,8 +2786,11 @@
       <c r="AR9" t="s">
         <v>83</v>
       </c>
+      <c r="AT9" t="s">
+        <v>94</v>
+      </c>
     </row>
-    <row r="10" ht="15" customHeight="1" spans="1:44" x14ac:dyDescent="0.25">
+    <row r="10" ht="15" customHeight="1" spans="1:46" x14ac:dyDescent="0.25">
       <c r="A10" t="s">
         <v>71</v>
       </c>
@@ -2801,7 +2807,7 @@
         <v>55</v>
       </c>
       <c r="F10" t="s">
-        <v>94</v>
+        <v>95</v>
       </c>
       <c r="G10" t="s">
         <v>77</v>
@@ -2831,7 +2837,7 @@
         <v>65</v>
       </c>
       <c r="P10" t="s">
-        <v>94</v>
+        <v>95</v>
       </c>
       <c r="Q10" t="s">
         <v>74</v>
@@ -2843,10 +2849,10 @@
         <v>64</v>
       </c>
       <c r="T10" t="s">
-        <v>94</v>
+        <v>95</v>
       </c>
       <c r="U10" t="s">
-        <v>95</v>
+        <v>96</v>
       </c>
       <c r="V10" t="s">
         <v>65</v>
@@ -2855,7 +2861,7 @@
         <v>74</v>
       </c>
       <c r="X10" t="s">
-        <v>95</v>
+        <v>96</v>
       </c>
       <c r="Y10" t="s">
         <v>73</v>
@@ -2891,7 +2897,7 @@
         <v>65</v>
       </c>
       <c r="AJ10" t="s">
-        <v>95</v>
+        <v>96</v>
       </c>
       <c r="AK10" t="s">
         <v>73</v>
@@ -2906,13 +2912,13 @@
         <v>92</v>
       </c>
       <c r="AO10" t="s">
-        <v>96</v>
+        <v>97</v>
       </c>
       <c r="AP10" t="s">
-        <v>97</v>
+        <v>98</v>
       </c>
       <c r="AQ10" t="s">
-        <v>98</v>
+        <v>99</v>
       </c>
     </row>
     <row r="11" ht="15" customHeight="1" spans="1:43" x14ac:dyDescent="0.25">
@@ -2941,7 +2947,7 @@
         <v>65</v>
       </c>
       <c r="I11" t="s">
-        <v>95</v>
+        <v>96</v>
       </c>
       <c r="J11" t="s">
         <v>64</v>
@@ -2989,13 +2995,13 @@
         <v>68</v>
       </c>
       <c r="Y11" t="s">
-        <v>95</v>
+        <v>96</v>
       </c>
       <c r="Z11" t="s">
-        <v>99</v>
+        <v>100</v>
       </c>
       <c r="AA11" t="s">
-        <v>95</v>
+        <v>96</v>
       </c>
       <c r="AB11" t="s">
         <v>78</v>
@@ -3010,7 +3016,7 @@
         <v>56</v>
       </c>
       <c r="AF11" t="s">
-        <v>99</v>
+        <v>100</v>
       </c>
       <c r="AG11" t="s">
         <v>68</v>
@@ -3019,7 +3025,7 @@
         <v>81</v>
       </c>
       <c r="AI11" t="s">
-        <v>99</v>
+        <v>100</v>
       </c>
       <c r="AJ11" t="s">
         <v>79</v>
@@ -3028,7 +3034,7 @@
         <v>86</v>
       </c>
       <c r="AL11" t="s">
-        <v>100</v>
+        <v>101</v>
       </c>
       <c r="AM11" t="s">
         <v>79</v>
@@ -3060,7 +3066,7 @@
         <v>65</v>
       </c>
       <c r="F12" t="s">
-        <v>95</v>
+        <v>96</v>
       </c>
       <c r="G12" t="s">
         <v>64</v>
@@ -3126,7 +3132,7 @@
         <v>91</v>
       </c>
       <c r="AB12" t="s">
-        <v>101</v>
+        <v>102</v>
       </c>
       <c r="AC12" t="s">
         <v>90</v>
@@ -3153,16 +3159,16 @@
         <v>80</v>
       </c>
       <c r="AK12" t="s">
-        <v>99</v>
+        <v>100</v>
       </c>
       <c r="AL12" t="s">
-        <v>102</v>
+        <v>103</v>
       </c>
       <c r="AM12" t="s">
-        <v>103</v>
+        <v>104</v>
       </c>
       <c r="AN12" t="s">
-        <v>104</v>
+        <v>105</v>
       </c>
       <c r="AO12" t="s">
         <v>83</v>
@@ -3182,7 +3188,7 @@
         <v>73</v>
       </c>
       <c r="D13" t="s">
-        <v>95</v>
+        <v>96</v>
       </c>
       <c r="E13" t="s">
         <v>73</v>
@@ -3251,16 +3257,16 @@
         <v>76</v>
       </c>
       <c r="AA13" t="s">
-        <v>99</v>
+        <v>100</v>
       </c>
       <c r="AB13" t="s">
-        <v>99</v>
+        <v>100</v>
       </c>
       <c r="AC13" t="s">
         <v>79</v>
       </c>
       <c r="AD13" t="s">
-        <v>100</v>
+        <v>101</v>
       </c>
       <c r="AE13" t="s">
         <v>80</v>
@@ -3275,7 +3281,7 @@
         <v>76</v>
       </c>
       <c r="AI13" t="s">
-        <v>96</v>
+        <v>97</v>
       </c>
       <c r="AJ13" t="s">
         <v>87</v>
@@ -3287,16 +3293,16 @@
         <v>82</v>
       </c>
       <c r="AM13" t="s">
-        <v>96</v>
+        <v>97</v>
       </c>
       <c r="AN13" t="s">
         <v>66</v>
       </c>
       <c r="AO13" t="s">
-        <v>97</v>
+        <v>98</v>
       </c>
       <c r="AP13" t="s">
-        <v>105</v>
+        <v>106</v>
       </c>
     </row>
     <row r="14" ht="15" customHeight="1" spans="1:42" x14ac:dyDescent="0.25">
@@ -3307,13 +3313,13 @@
         <v>64</v>
       </c>
       <c r="C14" t="s">
-        <v>95</v>
+        <v>96</v>
       </c>
       <c r="D14" t="s">
         <v>68</v>
       </c>
       <c r="E14" t="s">
-        <v>95</v>
+        <v>96</v>
       </c>
       <c r="F14" t="s">
         <v>90</v>
@@ -3325,13 +3331,13 @@
         <v>68</v>
       </c>
       <c r="I14" t="s">
-        <v>99</v>
+        <v>100</v>
       </c>
       <c r="J14" t="s">
-        <v>101</v>
+        <v>102</v>
       </c>
       <c r="K14" t="s">
-        <v>99</v>
+        <v>100</v>
       </c>
       <c r="L14" t="s">
         <v>79</v>
@@ -3346,7 +3352,7 @@
         <v>86</v>
       </c>
       <c r="P14" t="s">
-        <v>99</v>
+        <v>100</v>
       </c>
       <c r="Q14" t="s">
         <v>81</v>
@@ -3358,7 +3364,7 @@
         <v>81</v>
       </c>
       <c r="T14" t="s">
-        <v>99</v>
+        <v>100</v>
       </c>
       <c r="U14" t="s">
         <v>76</v>
@@ -3376,7 +3382,7 @@
         <v>81</v>
       </c>
       <c r="Z14" t="s">
-        <v>102</v>
+        <v>103</v>
       </c>
       <c r="AA14" t="s">
         <v>80</v>
@@ -3388,37 +3394,37 @@
         <v>81</v>
       </c>
       <c r="AD14" t="s">
-        <v>102</v>
+        <v>103</v>
       </c>
       <c r="AE14" t="s">
+        <v>101</v>
+      </c>
+      <c r="AF14" t="s">
+        <v>103</v>
+      </c>
+      <c r="AG14" t="s">
         <v>100</v>
       </c>
-      <c r="AF14" t="s">
-        <v>102</v>
-      </c>
-      <c r="AG14" t="s">
-        <v>99</v>
-      </c>
       <c r="AH14" t="s">
-        <v>106</v>
+        <v>107</v>
       </c>
       <c r="AI14" t="s">
-        <v>103</v>
+        <v>104</v>
       </c>
       <c r="AJ14" t="s">
-        <v>106</v>
+        <v>107</v>
       </c>
       <c r="AK14" t="s">
-        <v>106</v>
+        <v>107</v>
       </c>
       <c r="AL14" t="s">
         <v>61</v>
       </c>
       <c r="AM14" t="s">
-        <v>97</v>
+        <v>98</v>
       </c>
       <c r="AN14" t="s">
-        <v>107</v>
+        <v>108</v>
       </c>
       <c r="AO14" t="s">
         <v>60</v>
@@ -3426,7 +3432,7 @@
     </row>
     <row r="15" ht="15" customHeight="1" spans="1:41" x14ac:dyDescent="0.25">
       <c r="A15" t="s">
-        <v>95</v>
+        <v>96</v>
       </c>
       <c r="B15" t="s">
         <v>73</v>
@@ -3465,22 +3471,22 @@
         <v>86</v>
       </c>
       <c r="N15" t="s">
-        <v>101</v>
+        <v>102</v>
       </c>
       <c r="O15" t="s">
-        <v>99</v>
+        <v>100</v>
       </c>
       <c r="P15" t="s">
-        <v>108</v>
+        <v>109</v>
       </c>
       <c r="Q15" t="s">
-        <v>99</v>
+        <v>100</v>
       </c>
       <c r="R15" t="s">
         <v>86</v>
       </c>
       <c r="S15" t="s">
-        <v>99</v>
+        <v>100</v>
       </c>
       <c r="T15" t="s">
         <v>80</v>
@@ -3489,7 +3495,7 @@
         <v>87</v>
       </c>
       <c r="V15" t="s">
-        <v>99</v>
+        <v>100</v>
       </c>
       <c r="W15" t="s">
         <v>86</v>
@@ -3516,16 +3522,16 @@
         <v>64</v>
       </c>
       <c r="AE15" t="s">
-        <v>102</v>
+        <v>103</v>
       </c>
       <c r="AF15" t="s">
-        <v>94</v>
+        <v>95</v>
       </c>
       <c r="AG15" t="s">
         <v>76</v>
       </c>
       <c r="AH15" t="s">
-        <v>96</v>
+        <v>97</v>
       </c>
       <c r="AI15" t="s">
         <v>75</v>
@@ -3551,7 +3557,7 @@
         <v>68</v>
       </c>
       <c r="B16" t="s">
-        <v>95</v>
+        <v>96</v>
       </c>
       <c r="C16" t="s">
         <v>90</v>
@@ -3578,7 +3584,7 @@
         <v>80</v>
       </c>
       <c r="K16" t="s">
-        <v>106</v>
+        <v>107</v>
       </c>
       <c r="L16" t="s">
         <v>76</v>
@@ -3599,7 +3605,7 @@
         <v>76</v>
       </c>
       <c r="R16" t="s">
-        <v>99</v>
+        <v>100</v>
       </c>
       <c r="S16" t="s">
         <v>76</v>
@@ -3608,7 +3614,7 @@
         <v>76</v>
       </c>
       <c r="U16" t="s">
-        <v>106</v>
+        <v>107</v>
       </c>
       <c r="V16" t="s">
         <v>76</v>
@@ -3623,7 +3629,7 @@
         <v>87</v>
       </c>
       <c r="Z16" t="s">
-        <v>108</v>
+        <v>109</v>
       </c>
       <c r="AA16" t="s">
         <v>66</v>
@@ -3635,16 +3641,16 @@
         <v>87</v>
       </c>
       <c r="AD16" t="s">
-        <v>96</v>
+        <v>97</v>
       </c>
       <c r="AE16" t="s">
-        <v>96</v>
+        <v>97</v>
       </c>
       <c r="AF16" t="s">
-        <v>103</v>
+        <v>104</v>
       </c>
       <c r="AG16" t="s">
-        <v>100</v>
+        <v>101</v>
       </c>
       <c r="AH16" t="s">
         <v>66</v>
@@ -3659,10 +3665,10 @@
         <v>82</v>
       </c>
       <c r="AL16" t="s">
-        <v>99</v>
+        <v>100</v>
       </c>
       <c r="AN16" t="s">
-        <v>105</v>
+        <v>106</v>
       </c>
     </row>
     <row r="17" ht="15" customHeight="1" spans="1:40" x14ac:dyDescent="0.25">
@@ -3682,25 +3688,25 @@
         <v>79</v>
       </c>
       <c r="F17" t="s">
-        <v>99</v>
+        <v>100</v>
       </c>
       <c r="G17" t="s">
-        <v>99</v>
+        <v>100</v>
       </c>
       <c r="H17" t="s">
         <v>80</v>
       </c>
       <c r="I17" t="s">
-        <v>106</v>
+        <v>107</v>
       </c>
       <c r="J17" t="s">
         <v>76</v>
       </c>
       <c r="K17" t="s">
-        <v>109</v>
+        <v>110</v>
       </c>
       <c r="L17" t="s">
-        <v>106</v>
+        <v>107</v>
       </c>
       <c r="M17" t="s">
         <v>80</v>
@@ -3721,49 +3727,49 @@
         <v>87</v>
       </c>
       <c r="S17" t="s">
+        <v>103</v>
+      </c>
+      <c r="T17" t="s">
+        <v>101</v>
+      </c>
+      <c r="U17" t="s">
         <v>102</v>
-      </c>
-      <c r="T17" t="s">
-        <v>100</v>
-      </c>
-      <c r="U17" t="s">
-        <v>101</v>
       </c>
       <c r="V17" t="s">
         <v>87</v>
       </c>
       <c r="W17" t="s">
-        <v>99</v>
+        <v>100</v>
       </c>
       <c r="X17" t="s">
-        <v>109</v>
+        <v>110</v>
       </c>
       <c r="Y17" t="s">
-        <v>106</v>
+        <v>107</v>
       </c>
       <c r="Z17" t="s">
-        <v>103</v>
+        <v>104</v>
       </c>
       <c r="AA17" t="s">
-        <v>110</v>
+        <v>111</v>
       </c>
       <c r="AB17" t="s">
         <v>82</v>
       </c>
       <c r="AC17" t="s">
-        <v>102</v>
+        <v>103</v>
       </c>
       <c r="AD17" t="s">
-        <v>103</v>
+        <v>104</v>
       </c>
       <c r="AE17" t="s">
         <v>82</v>
       </c>
       <c r="AF17" t="s">
-        <v>110</v>
+        <v>111</v>
       </c>
       <c r="AG17" t="s">
-        <v>96</v>
+        <v>97</v>
       </c>
       <c r="AH17" t="s">
         <v>92</v>
@@ -3792,10 +3798,10 @@
         <v>78</v>
       </c>
       <c r="C18" t="s">
-        <v>101</v>
+        <v>102</v>
       </c>
       <c r="D18" t="s">
-        <v>101</v>
+        <v>102</v>
       </c>
       <c r="E18" t="s">
         <v>76</v>
@@ -3810,52 +3816,52 @@
         <v>76</v>
       </c>
       <c r="I18" t="s">
-        <v>100</v>
+        <v>101</v>
       </c>
       <c r="J18" t="s">
         <v>87</v>
       </c>
       <c r="K18" t="s">
-        <v>96</v>
+        <v>97</v>
       </c>
       <c r="L18" t="s">
-        <v>100</v>
+        <v>101</v>
       </c>
       <c r="M18" t="s">
-        <v>100</v>
+        <v>101</v>
       </c>
       <c r="N18" t="s">
         <v>87</v>
       </c>
       <c r="O18" t="s">
-        <v>102</v>
+        <v>103</v>
       </c>
       <c r="P18" t="s">
-        <v>103</v>
+        <v>104</v>
       </c>
       <c r="Q18" t="s">
         <v>66</v>
       </c>
       <c r="R18" t="s">
-        <v>100</v>
+        <v>101</v>
       </c>
       <c r="S18" t="s">
-        <v>103</v>
+        <v>104</v>
       </c>
       <c r="T18" t="s">
-        <v>103</v>
+        <v>104</v>
       </c>
       <c r="U18" t="s">
-        <v>96</v>
+        <v>97</v>
       </c>
       <c r="V18" t="s">
-        <v>96</v>
+        <v>97</v>
       </c>
       <c r="W18" t="s">
         <v>76</v>
       </c>
       <c r="X18" t="s">
-        <v>111</v>
+        <v>112</v>
       </c>
       <c r="Y18" t="s">
         <v>66</v>
@@ -3873,7 +3879,7 @@
         <v>66</v>
       </c>
       <c r="AD18" t="s">
-        <v>110</v>
+        <v>111</v>
       </c>
       <c r="AE18" t="s">
         <v>92</v>
@@ -3882,7 +3888,7 @@
         <v>75</v>
       </c>
       <c r="AG18" t="s">
-        <v>110</v>
+        <v>111</v>
       </c>
       <c r="AH18" t="s">
         <v>69</v>
@@ -3917,7 +3923,7 @@
         <v>86</v>
       </c>
       <c r="E19" t="s">
-        <v>106</v>
+        <v>107</v>
       </c>
       <c r="F19" t="s">
         <v>87</v>
@@ -3926,28 +3932,28 @@
         <v>87</v>
       </c>
       <c r="H19" t="s">
-        <v>106</v>
+        <v>107</v>
       </c>
       <c r="I19" t="s">
         <v>81</v>
       </c>
       <c r="J19" t="s">
-        <v>96</v>
+        <v>97</v>
       </c>
       <c r="K19" t="s">
         <v>82</v>
       </c>
       <c r="L19" t="s">
-        <v>102</v>
+        <v>103</v>
       </c>
       <c r="M19" t="s">
         <v>66</v>
       </c>
       <c r="N19" t="s">
-        <v>106</v>
+        <v>107</v>
       </c>
       <c r="O19" t="s">
-        <v>96</v>
+        <v>97</v>
       </c>
       <c r="P19" t="s">
         <v>75</v>
@@ -3956,10 +3962,10 @@
         <v>75</v>
       </c>
       <c r="R19" t="s">
-        <v>103</v>
+        <v>104</v>
       </c>
       <c r="S19" t="s">
-        <v>110</v>
+        <v>111</v>
       </c>
       <c r="T19" t="s">
         <v>82</v>
@@ -3971,25 +3977,25 @@
         <v>75</v>
       </c>
       <c r="W19" t="s">
-        <v>96</v>
+        <v>97</v>
       </c>
       <c r="X19" t="s">
-        <v>110</v>
+        <v>111</v>
       </c>
       <c r="Y19" t="s">
         <v>82</v>
       </c>
       <c r="Z19" t="s">
-        <v>104</v>
+        <v>105</v>
       </c>
       <c r="AA19" t="s">
-        <v>104</v>
+        <v>105</v>
       </c>
       <c r="AB19" t="s">
         <v>92</v>
       </c>
       <c r="AC19" t="s">
-        <v>103</v>
+        <v>104</v>
       </c>
       <c r="AD19" t="s">
         <v>60</v>
@@ -4004,36 +4010,39 @@
         <v>82</v>
       </c>
       <c r="AH19" t="s">
-        <v>104</v>
+        <v>105</v>
       </c>
       <c r="AI19" t="s">
-        <v>97</v>
+        <v>98</v>
       </c>
       <c r="AJ19" t="s">
         <v>93</v>
       </c>
       <c r="AK19" t="s">
-        <v>107</v>
+        <v>108</v>
+      </c>
+      <c r="AL19" t="s">
+        <v>98</v>
       </c>
     </row>
-    <row r="20" ht="15" customHeight="1" spans="1:37" x14ac:dyDescent="0.25">
+    <row r="20" ht="15" customHeight="1" spans="1:38" x14ac:dyDescent="0.25">
       <c r="A20" t="s">
+        <v>102</v>
+      </c>
+      <c r="B20" t="s">
+        <v>102</v>
+      </c>
+      <c r="C20" t="s">
+        <v>100</v>
+      </c>
+      <c r="D20" t="s">
+        <v>100</v>
+      </c>
+      <c r="E20" t="s">
         <v>101</v>
       </c>
-      <c r="B20" t="s">
-        <v>101</v>
-      </c>
-      <c r="C20" t="s">
-        <v>99</v>
-      </c>
-      <c r="D20" t="s">
-        <v>99</v>
-      </c>
-      <c r="E20" t="s">
-        <v>100</v>
-      </c>
       <c r="F20" t="s">
-        <v>102</v>
+        <v>103</v>
       </c>
       <c r="G20" t="s">
         <v>66</v>
@@ -4042,7 +4051,7 @@
         <v>78</v>
       </c>
       <c r="I20" t="s">
-        <v>96</v>
+        <v>97</v>
       </c>
       <c r="J20" t="s">
         <v>66</v>
@@ -4051,16 +4060,16 @@
         <v>61</v>
       </c>
       <c r="L20" t="s">
-        <v>96</v>
+        <v>97</v>
       </c>
       <c r="M20" t="s">
-        <v>103</v>
+        <v>104</v>
       </c>
       <c r="N20" t="s">
-        <v>96</v>
+        <v>97</v>
       </c>
       <c r="O20" t="s">
-        <v>103</v>
+        <v>104</v>
       </c>
       <c r="P20" t="s">
         <v>82</v>
@@ -4078,7 +4087,7 @@
         <v>61</v>
       </c>
       <c r="U20" t="s">
-        <v>110</v>
+        <v>111</v>
       </c>
       <c r="V20" t="s">
         <v>61</v>
@@ -4099,7 +4108,7 @@
         <v>69</v>
       </c>
       <c r="AB20" t="s">
-        <v>104</v>
+        <v>105</v>
       </c>
       <c r="AC20" t="s">
         <v>61</v>
@@ -4108,10 +4117,10 @@
         <v>83</v>
       </c>
       <c r="AE20" t="s">
-        <v>107</v>
+        <v>108</v>
       </c>
       <c r="AF20" t="s">
-        <v>96</v>
+        <v>97</v>
       </c>
       <c r="AG20" t="s">
         <v>92</v>
@@ -4120,13 +4129,13 @@
         <v>93</v>
       </c>
       <c r="AI20" t="s">
-        <v>105</v>
+        <v>106</v>
       </c>
       <c r="AJ20" t="s">
         <v>62</v>
       </c>
       <c r="AK20" t="s">
-        <v>112</v>
+        <v>113</v>
       </c>
     </row>
     <row r="21" ht="15" customHeight="1" spans="1:37" x14ac:dyDescent="0.25">
@@ -4134,25 +4143,25 @@
         <v>86</v>
       </c>
       <c r="B21" t="s">
-        <v>99</v>
+        <v>100</v>
       </c>
       <c r="C21" t="s">
-        <v>108</v>
+        <v>109</v>
       </c>
       <c r="D21" t="s">
-        <v>108</v>
+        <v>109</v>
       </c>
       <c r="E21" t="s">
-        <v>96</v>
+        <v>97</v>
       </c>
       <c r="F21" t="s">
         <v>73</v>
       </c>
       <c r="G21" t="s">
-        <v>110</v>
+        <v>111</v>
       </c>
       <c r="H21" t="s">
-        <v>96</v>
+        <v>97</v>
       </c>
       <c r="I21" t="s">
         <v>66</v>
@@ -4164,16 +4173,16 @@
         <v>60</v>
       </c>
       <c r="L21" t="s">
-        <v>103</v>
+        <v>104</v>
       </c>
       <c r="M21" t="s">
-        <v>110</v>
+        <v>111</v>
       </c>
       <c r="N21" t="s">
         <v>66</v>
       </c>
       <c r="O21" t="s">
-        <v>110</v>
+        <v>111</v>
       </c>
       <c r="P21" t="s">
         <v>61</v>
@@ -4206,31 +4215,31 @@
         <v>69</v>
       </c>
       <c r="Z21" t="s">
-        <v>96</v>
+        <v>97</v>
       </c>
       <c r="AA21" t="s">
-        <v>97</v>
+        <v>98</v>
       </c>
       <c r="AB21" t="s">
         <v>69</v>
       </c>
       <c r="AC21" t="s">
-        <v>104</v>
+        <v>105</v>
       </c>
       <c r="AD21" t="s">
-        <v>97</v>
+        <v>98</v>
       </c>
       <c r="AE21" t="s">
-        <v>97</v>
+        <v>98</v>
       </c>
       <c r="AF21" t="s">
-        <v>97</v>
+        <v>99</v>
       </c>
       <c r="AG21" t="s">
-        <v>104</v>
+        <v>105</v>
       </c>
       <c r="AH21" t="s">
-        <v>107</v>
+        <v>108</v>
       </c>
       <c r="AI21" t="s">
         <v>62</v>
@@ -4239,12 +4248,12 @@
         <v>61</v>
       </c>
       <c r="AK21" t="s">
-        <v>98</v>
+        <v>114</v>
       </c>
     </row>
     <row r="22" ht="15" customHeight="1" spans="1:37" x14ac:dyDescent="0.25">
       <c r="A22" t="s">
-        <v>99</v>
+        <v>100</v>
       </c>
       <c r="B22" t="s">
         <v>80</v>
@@ -4256,7 +4265,7 @@
         <v>76</v>
       </c>
       <c r="E22" t="s">
-        <v>111</v>
+        <v>112</v>
       </c>
       <c r="F22" t="s">
         <v>66</v>
@@ -4265,10 +4274,10 @@
         <v>75</v>
       </c>
       <c r="H22" t="s">
-        <v>103</v>
+        <v>104</v>
       </c>
       <c r="I22" t="s">
-        <v>103</v>
+        <v>104</v>
       </c>
       <c r="J22" t="s">
         <v>82</v>
@@ -4283,7 +4292,7 @@
         <v>60</v>
       </c>
       <c r="N22" t="s">
-        <v>103</v>
+        <v>104</v>
       </c>
       <c r="O22" t="s">
         <v>75</v>
@@ -4292,7 +4301,7 @@
         <v>60</v>
       </c>
       <c r="Q22" t="s">
-        <v>104</v>
+        <v>105</v>
       </c>
       <c r="R22" t="s">
         <v>60</v>
@@ -4301,7 +4310,7 @@
         <v>60</v>
       </c>
       <c r="T22" t="s">
-        <v>104</v>
+        <v>105</v>
       </c>
       <c r="U22" t="s">
         <v>61</v>
@@ -4310,19 +4319,19 @@
         <v>92</v>
       </c>
       <c r="W22" t="s">
-        <v>104</v>
+        <v>105</v>
       </c>
       <c r="X22" t="s">
-        <v>104</v>
+        <v>105</v>
       </c>
       <c r="Y22" t="s">
         <v>93</v>
       </c>
       <c r="Z22" t="s">
+        <v>115</v>
+      </c>
+      <c r="AA22" t="s">
         <v>113</v>
-      </c>
-      <c r="AA22" t="s">
-        <v>112</v>
       </c>
       <c r="AB22" t="s">
         <v>83</v>
@@ -4331,25 +4340,25 @@
         <v>69</v>
       </c>
       <c r="AD22" t="s">
-        <v>112</v>
+        <v>113</v>
       </c>
       <c r="AE22" t="s">
-        <v>105</v>
+        <v>106</v>
       </c>
       <c r="AF22" t="s">
-        <v>105</v>
+        <v>99</v>
       </c>
       <c r="AG22" t="s">
         <v>93</v>
       </c>
       <c r="AH22" t="s">
-        <v>97</v>
+        <v>98</v>
       </c>
       <c r="AI22" t="s">
+        <v>94</v>
+      </c>
+      <c r="AJ22" t="s">
         <v>114</v>
-      </c>
-      <c r="AJ22" t="s">
-        <v>98</v>
       </c>
     </row>
     <row r="23" ht="15" customHeight="1" spans="1:36" x14ac:dyDescent="0.25">
@@ -4366,10 +4375,10 @@
         <v>87</v>
       </c>
       <c r="E23" t="s">
-        <v>103</v>
+        <v>104</v>
       </c>
       <c r="F23" t="s">
-        <v>103</v>
+        <v>104</v>
       </c>
       <c r="G23" t="s">
         <v>82</v>
@@ -4384,31 +4393,34 @@
         <v>60</v>
       </c>
       <c r="K23" t="s">
-        <v>104</v>
+        <v>105</v>
       </c>
       <c r="L23" t="s">
         <v>61</v>
       </c>
       <c r="M23" t="s">
+        <v>116</v>
+      </c>
+      <c r="N23" t="s">
         <v>115</v>
-      </c>
-      <c r="N23" t="s">
-        <v>113</v>
       </c>
       <c r="O23" t="s">
         <v>61</v>
       </c>
       <c r="P23" t="s">
-        <v>104</v>
+        <v>105</v>
+      </c>
+      <c r="Q23" t="s">
+        <v>114</v>
       </c>
       <c r="R23" t="s">
-        <v>104</v>
+        <v>105</v>
       </c>
       <c r="S23" t="s">
         <v>92</v>
       </c>
       <c r="T23" t="s">
-        <v>113</v>
+        <v>115</v>
       </c>
       <c r="U23" t="s">
         <v>69</v>
@@ -4420,10 +4432,10 @@
         <v>69</v>
       </c>
       <c r="X23" t="s">
-        <v>102</v>
+        <v>103</v>
       </c>
       <c r="Y23" t="s">
-        <v>107</v>
+        <v>108</v>
       </c>
       <c r="Z23" t="s">
         <v>83</v>
@@ -4432,10 +4444,10 @@
         <v>62</v>
       </c>
       <c r="AB23" t="s">
-        <v>97</v>
+        <v>98</v>
       </c>
       <c r="AC23" t="s">
-        <v>107</v>
+        <v>108</v>
       </c>
       <c r="AD23" t="s">
         <v>62</v>
@@ -4444,13 +4456,13 @@
         <v>83</v>
       </c>
       <c r="AF23" t="s">
-        <v>112</v>
+        <v>113</v>
       </c>
       <c r="AG23" t="s">
-        <v>105</v>
+        <v>106</v>
       </c>
       <c r="AH23" t="s">
-        <v>105</v>
+        <v>106</v>
       </c>
     </row>
     <row r="24" ht="15" customHeight="1" spans="1:34" x14ac:dyDescent="0.25">
@@ -4458,16 +4470,16 @@
         <v>76</v>
       </c>
       <c r="B24" t="s">
-        <v>106</v>
+        <v>107</v>
       </c>
       <c r="C24" t="s">
-        <v>102</v>
+        <v>103</v>
       </c>
       <c r="D24" t="s">
-        <v>109</v>
+        <v>110</v>
       </c>
       <c r="E24" t="s">
-        <v>113</v>
+        <v>115</v>
       </c>
       <c r="F24" t="s">
         <v>82</v>
@@ -4482,13 +4494,13 @@
         <v>92</v>
       </c>
       <c r="J24" t="s">
-        <v>104</v>
+        <v>105</v>
       </c>
       <c r="K24" t="s">
-        <v>102</v>
+        <v>103</v>
       </c>
       <c r="L24" t="s">
-        <v>104</v>
+        <v>105</v>
       </c>
       <c r="M24" t="s">
         <v>82</v>
@@ -4497,10 +4509,10 @@
         <v>93</v>
       </c>
       <c r="O24" t="s">
-        <v>104</v>
+        <v>105</v>
       </c>
       <c r="P24" t="s">
-        <v>113</v>
+        <v>115</v>
       </c>
       <c r="R24" t="s">
         <v>69</v>
@@ -4524,22 +4536,22 @@
         <v>93</v>
       </c>
       <c r="Y24" t="s">
-        <v>105</v>
+        <v>106</v>
       </c>
       <c r="Z24" t="s">
-        <v>107</v>
+        <v>108</v>
       </c>
       <c r="AA24" t="s">
         <v>61</v>
       </c>
       <c r="AB24" t="s">
-        <v>112</v>
+        <v>113</v>
       </c>
       <c r="AC24" t="s">
-        <v>105</v>
+        <v>106</v>
       </c>
       <c r="AD24" t="s">
-        <v>98</v>
+        <v>114</v>
       </c>
       <c r="AE24" t="s">
         <v>61</v>
@@ -4551,7 +4563,7 @@
         <v>89</v>
       </c>
       <c r="AH24" t="s">
-        <v>114</v>
+        <v>94</v>
       </c>
     </row>
     <row r="25" ht="15" customHeight="1" spans="1:34" x14ac:dyDescent="0.25">
@@ -4559,10 +4571,10 @@
         <v>87</v>
       </c>
       <c r="B25" t="s">
-        <v>100</v>
+        <v>101</v>
       </c>
       <c r="C25" t="s">
-        <v>96</v>
+        <v>97</v>
       </c>
       <c r="D25" t="s">
         <v>75</v>
@@ -4580,7 +4592,7 @@
         <v>60</v>
       </c>
       <c r="I25" t="s">
-        <v>104</v>
+        <v>105</v>
       </c>
       <c r="J25" t="s">
         <v>83</v>
@@ -4595,7 +4607,7 @@
         <v>93</v>
       </c>
       <c r="N25" t="s">
-        <v>107</v>
+        <v>108</v>
       </c>
       <c r="O25" t="s">
         <v>83</v>
@@ -4610,25 +4622,25 @@
         <v>93</v>
       </c>
       <c r="T25" t="s">
-        <v>105</v>
+        <v>106</v>
       </c>
       <c r="U25" t="s">
-        <v>107</v>
+        <v>108</v>
       </c>
       <c r="V25" t="s">
-        <v>107</v>
+        <v>108</v>
       </c>
       <c r="W25" t="s">
-        <v>105</v>
+        <v>106</v>
       </c>
       <c r="X25" t="s">
-        <v>107</v>
+        <v>108</v>
       </c>
       <c r="Y25" t="s">
-        <v>116</v>
+        <v>117</v>
       </c>
       <c r="Z25" t="s">
-        <v>117</v>
+        <v>118</v>
       </c>
       <c r="AA25" t="s">
         <v>88</v>
@@ -4640,24 +4652,24 @@
         <v>89</v>
       </c>
       <c r="AE25" t="s">
-        <v>114</v>
+        <v>94</v>
       </c>
       <c r="AF25" t="s">
-        <v>114</v>
+        <v>94</v>
       </c>
       <c r="AH25" t="s">
-        <v>118</v>
+        <v>119</v>
       </c>
     </row>
     <row r="26" ht="15" customHeight="1" spans="1:34" x14ac:dyDescent="0.25">
       <c r="A26" t="s">
-        <v>100</v>
+        <v>101</v>
       </c>
       <c r="B26" t="s">
-        <v>109</v>
+        <v>110</v>
       </c>
       <c r="C26" t="s">
-        <v>111</v>
+        <v>112</v>
       </c>
       <c r="D26" t="s">
         <v>60</v>
@@ -4666,7 +4678,7 @@
         <v>92</v>
       </c>
       <c r="F26" t="s">
-        <v>104</v>
+        <v>105</v>
       </c>
       <c r="G26" t="s">
         <v>69</v>
@@ -4675,10 +4687,10 @@
         <v>92</v>
       </c>
       <c r="I26" t="s">
-        <v>115</v>
+        <v>116</v>
       </c>
       <c r="J26" t="s">
-        <v>107</v>
+        <v>108</v>
       </c>
       <c r="K26" t="s">
         <v>83</v>
@@ -4687,66 +4699,66 @@
         <v>93</v>
       </c>
       <c r="M26" t="s">
-        <v>116</v>
+        <v>117</v>
       </c>
       <c r="N26" t="s">
-        <v>97</v>
+        <v>98</v>
       </c>
       <c r="O26" t="s">
-        <v>107</v>
+        <v>108</v>
       </c>
       <c r="P26" t="s">
-        <v>107</v>
+        <v>108</v>
       </c>
       <c r="R26" t="s">
-        <v>112</v>
+        <v>113</v>
       </c>
       <c r="S26" t="s">
-        <v>107</v>
+        <v>108</v>
       </c>
       <c r="T26" t="s">
-        <v>117</v>
+        <v>118</v>
       </c>
       <c r="U26" t="s">
-        <v>97</v>
+        <v>98</v>
       </c>
       <c r="V26" t="s">
-        <v>97</v>
+        <v>98</v>
       </c>
       <c r="W26" t="s">
-        <v>114</v>
+        <v>94</v>
       </c>
       <c r="X26" t="s">
         <v>92</v>
       </c>
       <c r="Y26" t="s">
-        <v>112</v>
+        <v>113</v>
       </c>
       <c r="Z26" t="s">
-        <v>119</v>
+        <v>120</v>
       </c>
       <c r="AA26" t="s">
-        <v>98</v>
+        <v>114</v>
       </c>
       <c r="AB26" t="s">
-        <v>98</v>
+        <v>114</v>
       </c>
       <c r="AE26" t="s">
-        <v>98</v>
+        <v>114</v>
       </c>
       <c r="AF26" t="s">
-        <v>120</v>
+        <v>121</v>
       </c>
     </row>
     <row r="27" ht="15" customHeight="1" spans="1:32" x14ac:dyDescent="0.25">
       <c r="A27" t="s">
-        <v>102</v>
+        <v>103</v>
       </c>
       <c r="B27" t="s">
-        <v>96</v>
+        <v>97</v>
       </c>
       <c r="C27" t="s">
-        <v>103</v>
+        <v>104</v>
       </c>
       <c r="D27" t="s">
         <v>92</v>
@@ -4764,55 +4776,55 @@
         <v>66</v>
       </c>
       <c r="I27" t="s">
-        <v>107</v>
+        <v>108</v>
       </c>
       <c r="J27" t="s">
-        <v>105</v>
+        <v>106</v>
       </c>
       <c r="K27" t="s">
-        <v>97</v>
+        <v>98</v>
       </c>
       <c r="L27" t="s">
-        <v>107</v>
+        <v>108</v>
       </c>
       <c r="M27" t="s">
-        <v>112</v>
+        <v>113</v>
       </c>
       <c r="N27" t="s">
-        <v>105</v>
+        <v>106</v>
       </c>
       <c r="O27" t="s">
-        <v>97</v>
+        <v>98</v>
       </c>
       <c r="P27" t="s">
-        <v>117</v>
+        <v>118</v>
       </c>
       <c r="R27" t="s">
         <v>88</v>
       </c>
       <c r="S27" t="s">
-        <v>105</v>
+        <v>106</v>
       </c>
       <c r="T27" t="s">
-        <v>119</v>
+        <v>120</v>
       </c>
       <c r="U27" t="s">
         <v>88</v>
       </c>
       <c r="V27" t="s">
-        <v>105</v>
+        <v>106</v>
       </c>
       <c r="W27" t="s">
         <v>89</v>
       </c>
       <c r="X27" t="s">
-        <v>114</v>
+        <v>94</v>
       </c>
       <c r="Y27" t="s">
-        <v>120</v>
+        <v>121</v>
       </c>
       <c r="Z27" t="s">
-        <v>114</v>
+        <v>94</v>
       </c>
       <c r="AF27" t="s">
         <v>89</v>
@@ -4820,19 +4832,19 @@
     </row>
     <row r="28" ht="15" customHeight="1" spans="1:32" x14ac:dyDescent="0.25">
       <c r="A28" t="s">
-        <v>96</v>
+        <v>97</v>
       </c>
       <c r="B28" t="s">
-        <v>111</v>
+        <v>112</v>
       </c>
       <c r="C28" t="s">
-        <v>113</v>
+        <v>115</v>
       </c>
       <c r="D28" t="s">
-        <v>104</v>
+        <v>105</v>
       </c>
       <c r="E28" t="s">
-        <v>115</v>
+        <v>116</v>
       </c>
       <c r="F28" t="s">
         <v>81</v>
@@ -4841,52 +4853,52 @@
         <v>83</v>
       </c>
       <c r="H28" t="s">
-        <v>102</v>
+        <v>103</v>
       </c>
       <c r="I28" t="s">
-        <v>105</v>
+        <v>106</v>
       </c>
       <c r="J28" t="s">
-        <v>116</v>
+        <v>117</v>
       </c>
       <c r="K28" t="s">
-        <v>105</v>
+        <v>106</v>
       </c>
       <c r="L28" t="s">
-        <v>97</v>
+        <v>98</v>
       </c>
       <c r="M28" t="s">
         <v>61</v>
       </c>
       <c r="N28" t="s">
-        <v>112</v>
+        <v>113</v>
       </c>
       <c r="O28" t="s">
-        <v>112</v>
+        <v>113</v>
       </c>
       <c r="P28" t="s">
-        <v>119</v>
+        <v>120</v>
       </c>
       <c r="R28" t="s">
-        <v>114</v>
+        <v>94</v>
       </c>
       <c r="T28" t="s">
         <v>75</v>
       </c>
       <c r="U28" t="s">
-        <v>98</v>
+        <v>114</v>
       </c>
       <c r="V28" t="s">
-        <v>112</v>
+        <v>113</v>
       </c>
       <c r="X28" t="s">
         <v>89</v>
       </c>
       <c r="Y28" t="s">
-        <v>118</v>
+        <v>119</v>
       </c>
       <c r="Z28" t="s">
-        <v>120</v>
+        <v>121</v>
       </c>
     </row>
     <row r="29" ht="15" customHeight="1" spans="1:26" x14ac:dyDescent="0.25">
@@ -4894,10 +4906,10 @@
         <v>66</v>
       </c>
       <c r="B29" t="s">
-        <v>110</v>
+        <v>111</v>
       </c>
       <c r="C29" t="s">
-        <v>110</v>
+        <v>111</v>
       </c>
       <c r="D29" t="s">
         <v>69</v>
@@ -4909,22 +4921,22 @@
         <v>93</v>
       </c>
       <c r="G29" t="s">
-        <v>97</v>
+        <v>98</v>
       </c>
       <c r="H29" t="s">
         <v>93</v>
       </c>
       <c r="I29" t="s">
-        <v>112</v>
+        <v>113</v>
       </c>
       <c r="J29" t="s">
-        <v>112</v>
+        <v>113</v>
       </c>
       <c r="K29" t="s">
-        <v>116</v>
+        <v>117</v>
       </c>
       <c r="L29" t="s">
-        <v>112</v>
+        <v>113</v>
       </c>
       <c r="M29" t="s">
         <v>88</v>
@@ -4936,24 +4948,24 @@
         <v>82</v>
       </c>
       <c r="P29" t="s">
-        <v>114</v>
+        <v>94</v>
       </c>
       <c r="R29" t="s">
         <v>89</v>
       </c>
       <c r="T29" t="s">
-        <v>114</v>
+        <v>94</v>
       </c>
       <c r="U29" t="s">
         <v>89</v>
       </c>
       <c r="V29" t="s">
-        <v>114</v>
+        <v>94</v>
       </c>
     </row>
     <row r="30" ht="15" customHeight="1" spans="1:22" x14ac:dyDescent="0.25">
       <c r="A30" t="s">
-        <v>103</v>
+        <v>104</v>
       </c>
       <c r="B30" t="s">
         <v>82</v>
@@ -4962,16 +4974,16 @@
         <v>82</v>
       </c>
       <c r="D30" t="s">
-        <v>96</v>
+        <v>97</v>
       </c>
       <c r="E30" t="s">
-        <v>107</v>
+        <v>108</v>
       </c>
       <c r="F30" t="s">
-        <v>107</v>
+        <v>108</v>
       </c>
       <c r="G30" t="s">
-        <v>105</v>
+        <v>106</v>
       </c>
       <c r="H30" t="s">
         <v>83</v>
@@ -4980,22 +4992,22 @@
         <v>93</v>
       </c>
       <c r="J30" t="s">
-        <v>97</v>
+        <v>98</v>
       </c>
       <c r="K30" t="s">
         <v>62</v>
       </c>
       <c r="L30" t="s">
-        <v>114</v>
+        <v>94</v>
       </c>
       <c r="M30" t="s">
-        <v>114</v>
+        <v>94</v>
       </c>
       <c r="N30" t="s">
-        <v>114</v>
+        <v>94</v>
       </c>
       <c r="O30" t="s">
-        <v>114</v>
+        <v>94</v>
       </c>
       <c r="P30" t="s">
         <v>89</v>
@@ -5004,12 +5016,12 @@
         <v>89</v>
       </c>
       <c r="V30" t="s">
-        <v>98</v>
+        <v>114</v>
       </c>
     </row>
     <row r="31" ht="15" customHeight="1" spans="1:22" x14ac:dyDescent="0.25">
       <c r="A31" t="s">
-        <v>113</v>
+        <v>115</v>
       </c>
       <c r="B31" t="s">
         <v>61</v>
@@ -5021,40 +5033,43 @@
         <v>93</v>
       </c>
       <c r="E31" t="s">
-        <v>97</v>
+        <v>98</v>
       </c>
       <c r="F31" t="s">
-        <v>97</v>
+        <v>98</v>
       </c>
       <c r="G31" t="s">
-        <v>116</v>
+        <v>117</v>
       </c>
       <c r="H31" t="s">
-        <v>107</v>
+        <v>108</v>
       </c>
       <c r="I31" t="s">
-        <v>114</v>
+        <v>99</v>
       </c>
       <c r="J31" t="s">
-        <v>114</v>
+        <v>94</v>
       </c>
       <c r="K31" t="s">
-        <v>114</v>
+        <v>94</v>
       </c>
       <c r="L31" t="s">
-        <v>120</v>
+        <v>121</v>
       </c>
       <c r="M31" t="s">
         <v>89</v>
       </c>
       <c r="N31" t="s">
-        <v>98</v>
+        <v>114</v>
       </c>
       <c r="O31" t="s">
-        <v>120</v>
+        <v>121</v>
+      </c>
+      <c r="P31" t="s">
+        <v>106</v>
       </c>
     </row>
-    <row r="32" ht="15" customHeight="1" spans="1:15" x14ac:dyDescent="0.25">
+    <row r="32" ht="15" customHeight="1" spans="1:16" x14ac:dyDescent="0.25">
       <c r="A32" t="s">
         <v>60</v>
       </c>
@@ -5068,10 +5083,10 @@
         <v>83</v>
       </c>
       <c r="E32" t="s">
-        <v>105</v>
+        <v>106</v>
       </c>
       <c r="F32" t="s">
-        <v>105</v>
+        <v>106</v>
       </c>
       <c r="G32" t="s">
         <v>62</v>
@@ -5080,13 +5095,13 @@
         <v>82</v>
       </c>
       <c r="I32" t="s">
-        <v>118</v>
+        <v>119</v>
       </c>
       <c r="J32" t="s">
-        <v>98</v>
+        <v>114</v>
       </c>
       <c r="K32" t="s">
-        <v>120</v>
+        <v>121</v>
       </c>
       <c r="L32" t="s">
         <v>89</v>
@@ -5106,45 +5121,45 @@
         <v>92</v>
       </c>
       <c r="C33" t="s">
-        <v>104</v>
+        <v>105</v>
       </c>
       <c r="D33" t="s">
-        <v>107</v>
+        <v>108</v>
       </c>
       <c r="E33" t="s">
-        <v>112</v>
+        <v>113</v>
       </c>
       <c r="F33" t="s">
-        <v>112</v>
+        <v>113</v>
       </c>
       <c r="G33" t="s">
-        <v>104</v>
+        <v>105</v>
       </c>
       <c r="H33" t="s">
-        <v>114</v>
+        <v>94</v>
       </c>
     </row>
     <row r="34" ht="15" customHeight="1" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A34" t="s">
-        <v>104</v>
+        <v>105</v>
       </c>
       <c r="B34" t="s">
-        <v>104</v>
+        <v>105</v>
       </c>
       <c r="C34" t="s">
         <v>69</v>
       </c>
       <c r="D34" t="s">
-        <v>97</v>
+        <v>98</v>
       </c>
       <c r="E34" t="s">
-        <v>116</v>
+        <v>117</v>
       </c>
       <c r="F34" t="s">
         <v>61</v>
       </c>
       <c r="G34" t="s">
-        <v>114</v>
+        <v>94</v>
       </c>
       <c r="H34" t="s">
         <v>89</v>
@@ -5161,16 +5176,16 @@
         <v>93</v>
       </c>
       <c r="D35" t="s">
-        <v>105</v>
+        <v>106</v>
       </c>
       <c r="E35" t="s">
+        <v>94</v>
+      </c>
+      <c r="F35" t="s">
         <v>114</v>
       </c>
-      <c r="F35" t="s">
-        <v>98</v>
-      </c>
       <c r="G35" t="s">
-        <v>98</v>
+        <v>114</v>
       </c>
     </row>
     <row r="36" ht="15" customHeight="1" spans="1:7" x14ac:dyDescent="0.25">
@@ -5178,13 +5193,13 @@
         <v>93</v>
       </c>
       <c r="B36" t="s">
-        <v>115</v>
+        <v>116</v>
       </c>
       <c r="C36" t="s">
         <v>83</v>
       </c>
       <c r="D36" t="s">
-        <v>112</v>
+        <v>113</v>
       </c>
       <c r="E36" t="s">
         <v>89</v>
@@ -5198,10 +5213,10 @@
         <v>83</v>
       </c>
       <c r="B37" t="s">
-        <v>102</v>
+        <v>103</v>
       </c>
       <c r="C37" t="s">
-        <v>107</v>
+        <v>108</v>
       </c>
       <c r="D37" t="s">
         <v>62</v>
@@ -5209,58 +5224,58 @@
     </row>
     <row r="38" ht="15" customHeight="1" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A38" t="s">
-        <v>107</v>
+        <v>108</v>
       </c>
       <c r="B38" t="s">
-        <v>113</v>
+        <v>115</v>
       </c>
       <c r="C38" t="s">
-        <v>97</v>
+        <v>98</v>
       </c>
       <c r="D38" t="s">
-        <v>119</v>
+        <v>120</v>
       </c>
     </row>
     <row r="39" ht="15" customHeight="1" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A39" t="s">
-        <v>97</v>
+        <v>98</v>
       </c>
       <c r="B39" t="s">
         <v>93</v>
       </c>
       <c r="C39" t="s">
-        <v>105</v>
+        <v>106</v>
       </c>
       <c r="D39" t="s">
-        <v>114</v>
+        <v>94</v>
       </c>
     </row>
     <row r="40" ht="15" customHeight="1" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A40" t="s">
-        <v>105</v>
+        <v>106</v>
       </c>
       <c r="B40" t="s">
         <v>83</v>
       </c>
       <c r="C40" t="s">
-        <v>116</v>
+        <v>117</v>
       </c>
       <c r="D40" t="s">
-        <v>120</v>
+        <v>121</v>
       </c>
     </row>
     <row r="41" ht="15" customHeight="1" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A41" t="s">
-        <v>112</v>
+        <v>113</v>
       </c>
       <c r="B41" t="s">
-        <v>107</v>
+        <v>108</v>
       </c>
       <c r="C41" t="s">
-        <v>112</v>
+        <v>113</v>
       </c>
       <c r="D41" t="s">
-        <v>98</v>
+        <v>114</v>
       </c>
     </row>
     <row r="42" ht="15" customHeight="1" spans="1:4" x14ac:dyDescent="0.25">
@@ -5268,10 +5283,10 @@
         <v>62</v>
       </c>
       <c r="B42" t="s">
-        <v>97</v>
+        <v>98</v>
       </c>
       <c r="C42" t="s">
-        <v>117</v>
+        <v>118</v>
       </c>
       <c r="D42" t="s">
         <v>89</v>
@@ -5282,7 +5297,7 @@
         <v>88</v>
       </c>
       <c r="B43" t="s">
-        <v>105</v>
+        <v>106</v>
       </c>
       <c r="C43" t="s">
         <v>88</v>
@@ -5290,24 +5305,24 @@
     </row>
     <row r="44" ht="15" customHeight="1" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A44" t="s">
-        <v>114</v>
+        <v>94</v>
       </c>
       <c r="B44" t="s">
-        <v>112</v>
+        <v>113</v>
       </c>
       <c r="C44" t="s">
-        <v>114</v>
+        <v>94</v>
       </c>
     </row>
     <row r="45" ht="15" customHeight="1" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A45" t="s">
-        <v>98</v>
+        <v>114</v>
       </c>
       <c r="B45" t="s">
-        <v>116</v>
+        <v>117</v>
       </c>
       <c r="C45" t="s">
-        <v>120</v>
+        <v>121</v>
       </c>
     </row>
     <row r="46" ht="15" customHeight="1" spans="1:3" x14ac:dyDescent="0.25">
@@ -5318,12 +5333,12 @@
         <v>89</v>
       </c>
       <c r="C46" t="s">
-        <v>98</v>
+        <v>114</v>
       </c>
     </row>
     <row r="47" ht="15" customHeight="1" spans="1:3" x14ac:dyDescent="0.25">
       <c r="B47" t="s">
-        <v>118</v>
+        <v>119</v>
       </c>
       <c r="C47" t="s">
         <v>89</v>
@@ -5513,7 +5528,7 @@
         <v>74</v>
       </c>
       <c r="S3" t="s">
-        <v>94</v>
+        <v>95</v>
       </c>
       <c r="T3" t="s">
         <v>64</v>
@@ -5525,7 +5540,7 @@
         <v>73</v>
       </c>
       <c r="W3" t="s">
-        <v>95</v>
+        <v>96</v>
       </c>
       <c r="X3" t="s">
         <v>68</v>
@@ -5543,7 +5558,7 @@
         <v>79</v>
       </c>
       <c r="AC3" t="s">
-        <v>101</v>
+        <v>102</v>
       </c>
       <c r="AD3" t="s">
         <v>86</v>
@@ -5552,10 +5567,10 @@
         <v>81</v>
       </c>
       <c r="AF3" t="s">
-        <v>99</v>
+        <v>100</v>
       </c>
       <c r="AG3" t="s">
-        <v>108</v>
+        <v>109</v>
       </c>
       <c r="AH3" t="s">
         <v>80</v>
@@ -5567,34 +5582,34 @@
         <v>87</v>
       </c>
       <c r="AK3" t="s">
-        <v>106</v>
+        <v>107</v>
       </c>
       <c r="AL3" t="s">
-        <v>100</v>
+        <v>101</v>
       </c>
       <c r="AM3" t="s">
-        <v>109</v>
+        <v>110</v>
       </c>
       <c r="AN3" t="s">
-        <v>102</v>
+        <v>103</v>
       </c>
       <c r="AO3" t="s">
-        <v>96</v>
+        <v>97</v>
       </c>
       <c r="AP3" t="s">
-        <v>111</v>
+        <v>112</v>
       </c>
       <c r="AQ3" t="s">
         <v>66</v>
       </c>
       <c r="AR3" t="s">
-        <v>103</v>
+        <v>104</v>
       </c>
       <c r="AS3" t="s">
-        <v>113</v>
+        <v>115</v>
       </c>
       <c r="AT3" t="s">
-        <v>110</v>
+        <v>111</v>
       </c>
       <c r="AU3" t="s">
         <v>75</v>
@@ -5612,13 +5627,13 @@
         <v>92</v>
       </c>
       <c r="AZ3" t="s">
-        <v>104</v>
+        <v>105</v>
       </c>
       <c r="BA3" t="s">
         <v>69</v>
       </c>
       <c r="BB3" t="s">
-        <v>115</v>
+        <v>116</v>
       </c>
       <c r="BC3" t="s">
         <v>93</v>
@@ -5627,46 +5642,46 @@
         <v>83</v>
       </c>
       <c r="BE3" t="s">
-        <v>107</v>
+        <v>108</v>
       </c>
       <c r="BF3" t="s">
-        <v>97</v>
+        <v>98</v>
       </c>
       <c r="BG3" t="s">
-        <v>105</v>
+        <v>106</v>
       </c>
       <c r="BH3" t="s">
-        <v>116</v>
+        <v>117</v>
       </c>
       <c r="BI3" t="s">
-        <v>112</v>
+        <v>113</v>
       </c>
       <c r="BJ3" t="s">
         <v>62</v>
       </c>
       <c r="BK3" t="s">
-        <v>117</v>
+        <v>118</v>
       </c>
       <c r="BL3" t="s">
-        <v>119</v>
+        <v>120</v>
       </c>
       <c r="BM3" t="s">
         <v>88</v>
       </c>
       <c r="BN3" t="s">
+        <v>94</v>
+      </c>
+      <c r="BO3" t="s">
+        <v>121</v>
+      </c>
+      <c r="BP3" t="s">
         <v>114</v>
-      </c>
-      <c r="BO3" t="s">
-        <v>120</v>
-      </c>
-      <c r="BP3" t="s">
-        <v>98</v>
       </c>
       <c r="BQ3" t="s">
         <v>89</v>
       </c>
       <c r="BR3" t="s">
-        <v>118</v>
+        <v>119</v>
       </c>
     </row>
     <row r="4" ht="15" customHeight="1" spans="1:70" x14ac:dyDescent="0.25">
@@ -5692,7 +5707,7 @@
         <v>1</v>
       </c>
       <c r="H4" t="s">
-        <v>121</v>
+        <v>122</v>
       </c>
       <c r="I4" t="s">
         <v>0</v>
@@ -5710,7 +5725,7 @@
         <v>12</v>
       </c>
       <c r="N4" t="s">
-        <v>121</v>
+        <v>122</v>
       </c>
       <c r="O4" t="s">
         <v>14</v>
@@ -5731,7 +5746,7 @@
         <v>2</v>
       </c>
       <c r="U4" t="s">
-        <v>121</v>
+        <v>122</v>
       </c>
       <c r="V4" t="s">
         <v>12</v>
@@ -6657,7 +6672,7 @@
         <v>14</v>
       </c>
       <c r="BF8" t="s">
-        <v>34</v>
+        <v>6</v>
       </c>
       <c r="BG8" t="s">
         <v>32</v>
@@ -6827,7 +6842,7 @@
         <v>0</v>
       </c>
       <c r="BF9" t="s">
-        <v>6</v>
+        <v>34</v>
       </c>
       <c r="BG9" t="s">
         <v>34</v>
@@ -7232,7 +7247,7 @@
         <v>28</v>
       </c>
       <c r="T12" t="s">
-        <v>121</v>
+        <v>122</v>
       </c>
       <c r="V12" t="s">
         <v>1</v>
@@ -7629,7 +7644,7 @@
         <v>22</v>
       </c>
       <c r="BP14" t="s">
-        <v>42</v>
+        <v>9</v>
       </c>
       <c r="BQ14" t="s">
         <v>31</v>
@@ -7775,7 +7790,7 @@
         <v>9</v>
       </c>
       <c r="BP15" t="s">
-        <v>9</v>
+        <v>16</v>
       </c>
       <c r="BQ15" t="s">
         <v>15</v>
@@ -7813,7 +7828,7 @@
         <v>34</v>
       </c>
       <c r="R16" t="s">
-        <v>121</v>
+        <v>122</v>
       </c>
       <c r="T16" t="s">
         <v>19</v>
@@ -8156,7 +8171,7 @@
         <v>20</v>
       </c>
       <c r="BF18" t="s">
-        <v>31</v>
+        <v>30</v>
       </c>
       <c r="BG18" t="s">
         <v>8</v>
@@ -8287,7 +8302,7 @@
         <v>39</v>
       </c>
       <c r="BF19" t="s">
-        <v>30</v>
+        <v>37</v>
       </c>
       <c r="BG19" t="s">
         <v>13</v>
@@ -8411,7 +8426,7 @@
     </row>
     <row r="21" ht="15" customHeight="1" spans="1:69" x14ac:dyDescent="0.25">
       <c r="A21" t="s">
-        <v>121</v>
+        <v>122</v>
       </c>
       <c r="C21" t="s">
         <v>7</v>
@@ -8611,7 +8626,7 @@
         <v>9</v>
       </c>
       <c r="BN22" t="s">
-        <v>8</v>
+        <v>45</v>
       </c>
       <c r="BQ22" t="s">
         <v>22</v>
@@ -8709,7 +8724,7 @@
         <v>27</v>
       </c>
       <c r="BG23" t="s">
-        <v>31</v>
+        <v>15</v>
       </c>
       <c r="BI23" t="s">
         <v>24</v>
@@ -9191,7 +9206,7 @@
         <v>74</v>
       </c>
       <c r="S3" t="s">
-        <v>94</v>
+        <v>95</v>
       </c>
       <c r="T3" t="s">
         <v>64</v>
@@ -9203,7 +9218,7 @@
         <v>73</v>
       </c>
       <c r="W3" t="s">
-        <v>95</v>
+        <v>96</v>
       </c>
       <c r="X3" t="s">
         <v>68</v>
@@ -9221,7 +9236,7 @@
         <v>79</v>
       </c>
       <c r="AC3" t="s">
-        <v>101</v>
+        <v>102</v>
       </c>
       <c r="AD3" t="s">
         <v>86</v>
@@ -9230,10 +9245,10 @@
         <v>81</v>
       </c>
       <c r="AF3" t="s">
-        <v>99</v>
+        <v>100</v>
       </c>
       <c r="AG3" t="s">
-        <v>108</v>
+        <v>109</v>
       </c>
       <c r="AH3" t="s">
         <v>80</v>
@@ -9245,34 +9260,34 @@
         <v>87</v>
       </c>
       <c r="AK3" t="s">
-        <v>106</v>
+        <v>107</v>
       </c>
       <c r="AL3" t="s">
-        <v>100</v>
+        <v>101</v>
       </c>
       <c r="AM3" t="s">
-        <v>109</v>
+        <v>110</v>
       </c>
       <c r="AN3" t="s">
-        <v>102</v>
+        <v>103</v>
       </c>
       <c r="AO3" t="s">
-        <v>96</v>
+        <v>97</v>
       </c>
       <c r="AP3" t="s">
-        <v>111</v>
+        <v>112</v>
       </c>
       <c r="AQ3" t="s">
         <v>66</v>
       </c>
       <c r="AR3" t="s">
-        <v>103</v>
+        <v>104</v>
       </c>
       <c r="AS3" t="s">
-        <v>113</v>
+        <v>115</v>
       </c>
       <c r="AT3" t="s">
-        <v>110</v>
+        <v>111</v>
       </c>
       <c r="AU3" t="s">
         <v>75</v>
@@ -9290,13 +9305,13 @@
         <v>92</v>
       </c>
       <c r="AZ3" t="s">
-        <v>104</v>
+        <v>105</v>
       </c>
       <c r="BA3" t="s">
         <v>69</v>
       </c>
       <c r="BB3" t="s">
-        <v>115</v>
+        <v>116</v>
       </c>
       <c r="BC3" t="s">
         <v>93</v>
@@ -9305,906 +9320,906 @@
         <v>83</v>
       </c>
       <c r="BE3" t="s">
-        <v>107</v>
+        <v>108</v>
       </c>
       <c r="BF3" t="s">
-        <v>97</v>
+        <v>98</v>
       </c>
       <c r="BG3" t="s">
-        <v>105</v>
+        <v>106</v>
       </c>
       <c r="BH3" t="s">
-        <v>116</v>
+        <v>117</v>
       </c>
       <c r="BI3" t="s">
-        <v>112</v>
+        <v>113</v>
       </c>
       <c r="BJ3" t="s">
         <v>62</v>
       </c>
       <c r="BK3" t="s">
-        <v>117</v>
+        <v>118</v>
       </c>
       <c r="BL3" t="s">
-        <v>119</v>
+        <v>120</v>
       </c>
       <c r="BM3" t="s">
         <v>88</v>
       </c>
       <c r="BN3" t="s">
+        <v>94</v>
+      </c>
+      <c r="BO3" t="s">
+        <v>121</v>
+      </c>
+      <c r="BP3" t="s">
         <v>114</v>
-      </c>
-      <c r="BO3" t="s">
-        <v>120</v>
-      </c>
-      <c r="BP3" t="s">
-        <v>98</v>
       </c>
       <c r="BQ3" t="s">
         <v>89</v>
       </c>
       <c r="BR3" t="s">
-        <v>118</v>
+        <v>119</v>
       </c>
     </row>
     <row r="4" ht="15" customHeight="1" spans="1:70" x14ac:dyDescent="0.25">
       <c r="A4" t="s">
-        <v>122</v>
+        <v>123</v>
       </c>
       <c r="B4" t="s">
-        <v>123</v>
+        <v>124</v>
       </c>
       <c r="C4" t="s">
-        <v>124</v>
+        <v>125</v>
       </c>
       <c r="D4" t="s">
-        <v>125</v>
+        <v>126</v>
       </c>
       <c r="E4" t="s">
-        <v>126</v>
+        <v>127</v>
       </c>
       <c r="F4" t="s">
-        <v>127</v>
+        <v>128</v>
       </c>
       <c r="G4" t="s">
-        <v>128</v>
+        <v>129</v>
       </c>
       <c r="H4" t="s">
-        <v>129</v>
+        <v>130</v>
       </c>
       <c r="I4" t="s">
-        <v>130</v>
+        <v>131</v>
       </c>
       <c r="J4" t="s">
-        <v>131</v>
+        <v>132</v>
       </c>
       <c r="K4" t="s">
-        <v>132</v>
+        <v>133</v>
       </c>
       <c r="L4" t="s">
-        <v>133</v>
+        <v>134</v>
       </c>
       <c r="M4" t="s">
-        <v>134</v>
+        <v>135</v>
       </c>
       <c r="N4" t="s">
-        <v>135</v>
+        <v>136</v>
       </c>
       <c r="O4" t="s">
-        <v>136</v>
+        <v>137</v>
       </c>
       <c r="P4" t="s">
-        <v>137</v>
+        <v>138</v>
       </c>
       <c r="Q4" t="s">
-        <v>138</v>
+        <v>139</v>
       </c>
       <c r="R4" t="s">
-        <v>139</v>
+        <v>140</v>
       </c>
       <c r="S4" t="s">
-        <v>140</v>
+        <v>141</v>
       </c>
       <c r="T4" t="s">
-        <v>141</v>
+        <v>142</v>
       </c>
       <c r="U4" t="s">
-        <v>142</v>
+        <v>143</v>
       </c>
       <c r="V4" t="s">
-        <v>143</v>
+        <v>144</v>
       </c>
       <c r="W4" t="s">
-        <v>144</v>
+        <v>145</v>
       </c>
       <c r="X4" t="s">
-        <v>145</v>
+        <v>146</v>
       </c>
       <c r="Y4" t="s">
-        <v>146</v>
+        <v>147</v>
       </c>
       <c r="Z4" t="s">
-        <v>147</v>
+        <v>148</v>
       </c>
       <c r="AA4" t="s">
-        <v>148</v>
+        <v>149</v>
       </c>
       <c r="AB4" t="s">
-        <v>149</v>
+        <v>150</v>
       </c>
       <c r="AC4" t="s">
-        <v>150</v>
+        <v>151</v>
       </c>
       <c r="AD4" t="s">
-        <v>151</v>
+        <v>152</v>
       </c>
       <c r="AE4" t="s">
-        <v>152</v>
+        <v>153</v>
       </c>
       <c r="AF4" t="s">
-        <v>153</v>
+        <v>154</v>
       </c>
       <c r="AG4" t="s">
-        <v>154</v>
+        <v>155</v>
       </c>
       <c r="AH4" t="s">
-        <v>155</v>
+        <v>156</v>
       </c>
       <c r="AI4" t="s">
-        <v>156</v>
+        <v>157</v>
       </c>
       <c r="AJ4" t="s">
-        <v>157</v>
+        <v>158</v>
       </c>
       <c r="AK4" t="s">
-        <v>158</v>
+        <v>159</v>
       </c>
       <c r="AL4" t="s">
-        <v>159</v>
+        <v>160</v>
       </c>
       <c r="AM4" t="s">
-        <v>160</v>
+        <v>161</v>
       </c>
       <c r="AN4" t="s">
-        <v>161</v>
+        <v>162</v>
       </c>
       <c r="AO4" t="s">
-        <v>162</v>
+        <v>163</v>
       </c>
       <c r="AP4" t="s">
-        <v>163</v>
+        <v>164</v>
       </c>
       <c r="AQ4" t="s">
-        <v>164</v>
+        <v>165</v>
       </c>
       <c r="AR4" t="s">
-        <v>165</v>
+        <v>166</v>
       </c>
       <c r="AS4" t="s">
-        <v>166</v>
+        <v>167</v>
       </c>
       <c r="AT4" t="s">
-        <v>167</v>
+        <v>168</v>
       </c>
       <c r="AU4" t="s">
-        <v>168</v>
+        <v>169</v>
       </c>
       <c r="AV4" t="s">
-        <v>169</v>
+        <v>170</v>
       </c>
       <c r="AW4" t="s">
-        <v>170</v>
+        <v>171</v>
       </c>
       <c r="AX4" t="s">
-        <v>171</v>
+        <v>172</v>
       </c>
       <c r="AY4" t="s">
-        <v>172</v>
+        <v>173</v>
       </c>
       <c r="AZ4" t="s">
-        <v>173</v>
+        <v>174</v>
       </c>
       <c r="BA4" t="s">
-        <v>174</v>
+        <v>175</v>
       </c>
       <c r="BB4" t="s">
-        <v>175</v>
+        <v>176</v>
       </c>
       <c r="BC4" t="s">
-        <v>176</v>
+        <v>177</v>
       </c>
       <c r="BD4" t="s">
-        <v>177</v>
+        <v>178</v>
       </c>
       <c r="BE4" t="s">
-        <v>178</v>
+        <v>179</v>
       </c>
       <c r="BF4" t="s">
-        <v>179</v>
+        <v>180</v>
       </c>
       <c r="BG4" t="s">
-        <v>180</v>
+        <v>181</v>
       </c>
       <c r="BH4" t="s">
-        <v>181</v>
+        <v>182</v>
       </c>
       <c r="BI4" t="s">
-        <v>182</v>
+        <v>183</v>
       </c>
       <c r="BJ4" t="s">
-        <v>183</v>
+        <v>184</v>
       </c>
       <c r="BK4" t="s">
-        <v>184</v>
+        <v>185</v>
       </c>
       <c r="BL4" t="s">
-        <v>185</v>
+        <v>186</v>
       </c>
       <c r="BM4" t="s">
-        <v>186</v>
+        <v>187</v>
       </c>
       <c r="BN4" t="s">
-        <v>187</v>
+        <v>188</v>
       </c>
       <c r="BO4" t="s">
-        <v>188</v>
+        <v>189</v>
       </c>
       <c r="BP4" t="s">
-        <v>189</v>
+        <v>190</v>
       </c>
       <c r="BQ4" t="s">
-        <v>190</v>
+        <v>191</v>
       </c>
       <c r="BR4" t="s">
-        <v>191</v>
+        <v>192</v>
       </c>
     </row>
     <row r="5" ht="15" customHeight="1" spans="1:70" x14ac:dyDescent="0.25">
       <c r="A5" t="s">
-        <v>192</v>
+        <v>193</v>
       </c>
       <c r="C5" t="s">
-        <v>193</v>
+        <v>194</v>
       </c>
       <c r="E5" t="s">
-        <v>194</v>
+        <v>195</v>
       </c>
       <c r="F5" t="s">
-        <v>195</v>
+        <v>196</v>
       </c>
       <c r="G5" t="s">
-        <v>196</v>
+        <v>197</v>
       </c>
       <c r="H5" t="s">
-        <v>197</v>
+        <v>198</v>
       </c>
       <c r="J5" t="s">
-        <v>198</v>
+        <v>199</v>
       </c>
       <c r="K5" t="s">
+        <v>200</v>
+      </c>
+      <c r="L5" t="s">
+        <v>201</v>
+      </c>
+      <c r="M5" t="s">
+        <v>202</v>
+      </c>
+      <c r="O5" t="s">
+        <v>203</v>
+      </c>
+      <c r="Q5" t="s">
+        <v>204</v>
+      </c>
+      <c r="R5" t="s">
+        <v>205</v>
+      </c>
+      <c r="T5" t="s">
+        <v>206</v>
+      </c>
+      <c r="V5" t="s">
+        <v>207</v>
+      </c>
+      <c r="W5" t="s">
+        <v>208</v>
+      </c>
+      <c r="X5" t="s">
+        <v>209</v>
+      </c>
+      <c r="Y5" t="s">
+        <v>210</v>
+      </c>
+      <c r="Z5" t="s">
+        <v>211</v>
+      </c>
+      <c r="AA5" t="s">
+        <v>212</v>
+      </c>
+      <c r="AB5" t="s">
+        <v>213</v>
+      </c>
+      <c r="AC5" t="s">
+        <v>214</v>
+      </c>
+      <c r="AD5" t="s">
+        <v>215</v>
+      </c>
+      <c r="AE5" t="s">
+        <v>216</v>
+      </c>
+      <c r="AF5" t="s">
+        <v>217</v>
+      </c>
+      <c r="AH5" t="s">
+        <v>218</v>
+      </c>
+      <c r="AI5" t="s">
+        <v>219</v>
+      </c>
+      <c r="AJ5" t="s">
+        <v>220</v>
+      </c>
+      <c r="AK5" t="s">
+        <v>221</v>
+      </c>
+      <c r="AL5" t="s">
+        <v>222</v>
+      </c>
+      <c r="AN5" t="s">
+        <v>223</v>
+      </c>
+      <c r="AO5" t="s">
+        <v>223</v>
+      </c>
+      <c r="AQ5" t="s">
+        <v>224</v>
+      </c>
+      <c r="AR5" t="s">
+        <v>225</v>
+      </c>
+      <c r="AS5" t="s">
+        <v>223</v>
+      </c>
+      <c r="AT5" t="s">
+        <v>226</v>
+      </c>
+      <c r="AU5" t="s">
         <v>199</v>
       </c>
-      <c r="L5" t="s">
-        <v>200</v>
-      </c>
-      <c r="M5" t="s">
-        <v>201</v>
-      </c>
-      <c r="O5" t="s">
-        <v>202</v>
-      </c>
-      <c r="Q5" t="s">
-        <v>203</v>
-      </c>
-      <c r="R5" t="s">
-        <v>204</v>
-      </c>
-      <c r="T5" t="s">
-        <v>205</v>
-      </c>
-      <c r="V5" t="s">
-        <v>206</v>
-      </c>
-      <c r="W5" t="s">
-        <v>207</v>
-      </c>
-      <c r="X5" t="s">
-        <v>208</v>
-      </c>
-      <c r="Y5" t="s">
-        <v>209</v>
-      </c>
-      <c r="Z5" t="s">
-        <v>210</v>
-      </c>
-      <c r="AA5" t="s">
-        <v>211</v>
-      </c>
-      <c r="AB5" t="s">
-        <v>212</v>
-      </c>
-      <c r="AC5" t="s">
-        <v>213</v>
-      </c>
-      <c r="AD5" t="s">
-        <v>214</v>
-      </c>
-      <c r="AE5" t="s">
-        <v>215</v>
-      </c>
-      <c r="AF5" t="s">
-        <v>216</v>
-      </c>
-      <c r="AH5" t="s">
-        <v>217</v>
-      </c>
-      <c r="AI5" t="s">
-        <v>218</v>
-      </c>
-      <c r="AJ5" t="s">
-        <v>219</v>
-      </c>
-      <c r="AK5" t="s">
-        <v>220</v>
-      </c>
-      <c r="AL5" t="s">
-        <v>221</v>
-      </c>
-      <c r="AN5" t="s">
-        <v>222</v>
-      </c>
-      <c r="AO5" t="s">
-        <v>222</v>
-      </c>
-      <c r="AQ5" t="s">
-        <v>223</v>
-      </c>
-      <c r="AR5" t="s">
-        <v>224</v>
-      </c>
-      <c r="AS5" t="s">
-        <v>222</v>
-      </c>
-      <c r="AT5" t="s">
-        <v>225</v>
-      </c>
-      <c r="AU5" t="s">
-        <v>198</v>
-      </c>
       <c r="AV5" t="s">
-        <v>226</v>
+        <v>227</v>
       </c>
       <c r="AW5" t="s">
-        <v>227</v>
+        <v>228</v>
       </c>
       <c r="AX5" t="s">
-        <v>228</v>
+        <v>229</v>
       </c>
       <c r="AY5" t="s">
-        <v>229</v>
+        <v>230</v>
       </c>
       <c r="AZ5" t="s">
-        <v>230</v>
+        <v>231</v>
       </c>
       <c r="BA5" t="s">
-        <v>231</v>
+        <v>232</v>
       </c>
       <c r="BC5" t="s">
-        <v>232</v>
+        <v>233</v>
       </c>
       <c r="BD5" t="s">
-        <v>233</v>
+        <v>234</v>
       </c>
       <c r="BE5" t="s">
-        <v>234</v>
+        <v>235</v>
       </c>
       <c r="BF5" t="s">
-        <v>235</v>
+        <v>236</v>
       </c>
       <c r="BG5" t="s">
-        <v>236</v>
+        <v>237</v>
       </c>
       <c r="BH5" t="s">
-        <v>237</v>
+        <v>238</v>
       </c>
       <c r="BI5" t="s">
-        <v>238</v>
+        <v>239</v>
       </c>
       <c r="BJ5" t="s">
-        <v>239</v>
+        <v>240</v>
       </c>
       <c r="BM5" t="s">
-        <v>240</v>
+        <v>241</v>
       </c>
       <c r="BN5" t="s">
-        <v>241</v>
+        <v>242</v>
       </c>
       <c r="BO5" t="s">
-        <v>242</v>
+        <v>243</v>
       </c>
       <c r="BP5" t="s">
-        <v>243</v>
+        <v>244</v>
       </c>
       <c r="BQ5" t="s">
-        <v>244</v>
+        <v>245</v>
       </c>
     </row>
     <row r="6" ht="15" customHeight="1" spans="1:69" x14ac:dyDescent="0.25">
       <c r="A6" t="s">
-        <v>245</v>
+        <v>246</v>
       </c>
       <c r="C6" t="s">
-        <v>246</v>
+        <v>247</v>
       </c>
       <c r="E6" t="s">
-        <v>247</v>
+        <v>248</v>
       </c>
       <c r="F6" t="s">
-        <v>248</v>
+        <v>249</v>
       </c>
       <c r="H6" t="s">
-        <v>249</v>
+        <v>250</v>
       </c>
       <c r="J6" t="s">
-        <v>250</v>
+        <v>251</v>
       </c>
       <c r="K6" t="s">
-        <v>251</v>
+        <v>252</v>
       </c>
       <c r="M6" t="s">
-        <v>252</v>
+        <v>253</v>
       </c>
       <c r="O6" t="s">
-        <v>253</v>
+        <v>254</v>
       </c>
       <c r="Q6" t="s">
-        <v>254</v>
+        <v>255</v>
       </c>
       <c r="R6" t="s">
-        <v>255</v>
+        <v>256</v>
       </c>
       <c r="T6" t="s">
-        <v>256</v>
+        <v>257</v>
       </c>
       <c r="V6" t="s">
-        <v>257</v>
+        <v>258</v>
       </c>
       <c r="W6" t="s">
-        <v>258</v>
+        <v>259</v>
       </c>
       <c r="X6" t="s">
-        <v>259</v>
+        <v>260</v>
       </c>
       <c r="Z6" t="s">
-        <v>260</v>
+        <v>261</v>
       </c>
       <c r="AA6" t="s">
-        <v>261</v>
+        <v>262</v>
       </c>
       <c r="AB6" t="s">
-        <v>262</v>
+        <v>263</v>
       </c>
       <c r="AD6" t="s">
-        <v>263</v>
+        <v>264</v>
       </c>
       <c r="AE6" t="s">
-        <v>264</v>
+        <v>265</v>
       </c>
       <c r="AF6" t="s">
-        <v>265</v>
+        <v>266</v>
       </c>
       <c r="AH6" t="s">
-        <v>266</v>
+        <v>267</v>
       </c>
       <c r="AI6" t="s">
-        <v>267</v>
+        <v>268</v>
       </c>
       <c r="AJ6" t="s">
-        <v>268</v>
+        <v>269</v>
       </c>
       <c r="AK6" t="s">
-        <v>269</v>
+        <v>270</v>
       </c>
       <c r="AL6" t="s">
-        <v>270</v>
+        <v>271</v>
       </c>
       <c r="AN6" t="s">
-        <v>271</v>
+        <v>272</v>
       </c>
       <c r="AO6" t="s">
-        <v>272</v>
+        <v>273</v>
       </c>
       <c r="AQ6" t="s">
-        <v>273</v>
+        <v>274</v>
       </c>
       <c r="AR6" t="s">
-        <v>274</v>
+        <v>275</v>
       </c>
       <c r="AS6" t="s">
-        <v>275</v>
+        <v>276</v>
       </c>
       <c r="AT6" t="s">
-        <v>276</v>
+        <v>277</v>
       </c>
       <c r="AU6" t="s">
-        <v>277</v>
+        <v>278</v>
       </c>
       <c r="AV6" t="s">
-        <v>278</v>
+        <v>279</v>
       </c>
       <c r="AW6" t="s">
-        <v>222</v>
+        <v>223</v>
       </c>
       <c r="AX6" t="s">
-        <v>279</v>
+        <v>280</v>
       </c>
       <c r="AY6" t="s">
-        <v>280</v>
+        <v>281</v>
       </c>
       <c r="AZ6" t="s">
-        <v>281</v>
+        <v>282</v>
       </c>
       <c r="BA6" t="s">
-        <v>282</v>
+        <v>283</v>
       </c>
       <c r="BC6" t="s">
-        <v>283</v>
+        <v>284</v>
       </c>
       <c r="BD6" t="s">
-        <v>284</v>
+        <v>285</v>
       </c>
       <c r="BE6" t="s">
-        <v>285</v>
+        <v>286</v>
       </c>
       <c r="BF6" t="s">
-        <v>286</v>
+        <v>287</v>
       </c>
       <c r="BG6" t="s">
-        <v>287</v>
+        <v>288</v>
       </c>
       <c r="BI6" t="s">
-        <v>288</v>
+        <v>289</v>
       </c>
       <c r="BJ6" t="s">
-        <v>289</v>
+        <v>290</v>
       </c>
       <c r="BN6" t="s">
-        <v>290</v>
+        <v>291</v>
       </c>
       <c r="BP6" t="s">
-        <v>291</v>
+        <v>292</v>
       </c>
       <c r="BQ6" t="s">
-        <v>292</v>
+        <v>293</v>
       </c>
     </row>
     <row r="7" ht="15" customHeight="1" spans="1:69" x14ac:dyDescent="0.25">
       <c r="A7" t="s">
-        <v>293</v>
+        <v>294</v>
       </c>
       <c r="C7" t="s">
-        <v>294</v>
+        <v>295</v>
       </c>
       <c r="E7" t="s">
-        <v>295</v>
+        <v>296</v>
       </c>
       <c r="F7" t="s">
-        <v>296</v>
+        <v>297</v>
       </c>
       <c r="H7" t="s">
-        <v>297</v>
+        <v>298</v>
       </c>
       <c r="J7" t="s">
-        <v>298</v>
+        <v>299</v>
       </c>
       <c r="K7" t="s">
-        <v>299</v>
+        <v>300</v>
       </c>
       <c r="M7" t="s">
-        <v>300</v>
+        <v>301</v>
       </c>
       <c r="O7" t="s">
-        <v>301</v>
+        <v>302</v>
       </c>
       <c r="Q7" t="s">
-        <v>302</v>
+        <v>303</v>
       </c>
       <c r="R7" t="s">
-        <v>303</v>
+        <v>304</v>
       </c>
       <c r="T7" t="s">
-        <v>304</v>
+        <v>305</v>
       </c>
       <c r="V7" t="s">
-        <v>305</v>
+        <v>306</v>
       </c>
       <c r="X7" t="s">
-        <v>306</v>
+        <v>307</v>
       </c>
       <c r="Z7" t="s">
-        <v>307</v>
+        <v>308</v>
       </c>
       <c r="AA7" t="s">
-        <v>308</v>
+        <v>309</v>
       </c>
       <c r="AB7" t="s">
-        <v>309</v>
+        <v>310</v>
       </c>
       <c r="AD7" t="s">
-        <v>310</v>
+        <v>311</v>
       </c>
       <c r="AE7" t="s">
-        <v>311</v>
+        <v>312</v>
       </c>
       <c r="AF7" t="s">
-        <v>312</v>
+        <v>313</v>
       </c>
       <c r="AH7" t="s">
-        <v>313</v>
+        <v>314</v>
       </c>
       <c r="AI7" t="s">
-        <v>314</v>
+        <v>315</v>
       </c>
       <c r="AJ7" t="s">
-        <v>315</v>
+        <v>316</v>
       </c>
       <c r="AN7" t="s">
-        <v>316</v>
+        <v>317</v>
       </c>
       <c r="AO7" t="s">
-        <v>317</v>
+        <v>318</v>
       </c>
       <c r="AQ7" t="s">
-        <v>318</v>
+        <v>319</v>
       </c>
       <c r="AR7" t="s">
-        <v>319</v>
+        <v>320</v>
       </c>
       <c r="AU7" t="s">
-        <v>320</v>
+        <v>321</v>
       </c>
       <c r="AV7" t="s">
-        <v>321</v>
+        <v>322</v>
       </c>
       <c r="AW7" t="s">
-        <v>322</v>
+        <v>323</v>
       </c>
       <c r="AX7" t="s">
-        <v>323</v>
+        <v>324</v>
       </c>
       <c r="AY7" t="s">
-        <v>324</v>
+        <v>325</v>
       </c>
       <c r="AZ7" t="s">
-        <v>325</v>
+        <v>326</v>
       </c>
       <c r="BA7" t="s">
-        <v>326</v>
+        <v>327</v>
       </c>
       <c r="BC7" t="s">
-        <v>327</v>
+        <v>328</v>
       </c>
       <c r="BD7" t="s">
-        <v>328</v>
+        <v>329</v>
       </c>
       <c r="BE7" t="s">
-        <v>329</v>
+        <v>330</v>
       </c>
       <c r="BF7" t="s">
-        <v>330</v>
+        <v>331</v>
       </c>
       <c r="BG7" t="s">
-        <v>331</v>
+        <v>332</v>
       </c>
       <c r="BI7" t="s">
-        <v>332</v>
+        <v>333</v>
       </c>
       <c r="BN7" t="s">
-        <v>333</v>
+        <v>334</v>
       </c>
       <c r="BP7" t="s">
-        <v>334</v>
+        <v>335</v>
       </c>
       <c r="BQ7" t="s">
-        <v>335</v>
+        <v>336</v>
       </c>
     </row>
     <row r="8" ht="15" customHeight="1" spans="1:69" x14ac:dyDescent="0.25">
       <c r="A8" t="s">
-        <v>336</v>
+        <v>337</v>
       </c>
       <c r="C8" t="s">
-        <v>337</v>
+        <v>338</v>
       </c>
       <c r="E8" t="s">
-        <v>338</v>
+        <v>339</v>
       </c>
       <c r="F8" t="s">
-        <v>339</v>
+        <v>340</v>
       </c>
       <c r="H8" t="s">
-        <v>340</v>
+        <v>341</v>
       </c>
       <c r="K8" t="s">
-        <v>341</v>
+        <v>342</v>
       </c>
       <c r="O8" t="s">
-        <v>342</v>
+        <v>343</v>
       </c>
       <c r="Q8" t="s">
-        <v>343</v>
+        <v>344</v>
       </c>
       <c r="R8" t="s">
-        <v>344</v>
+        <v>345</v>
       </c>
       <c r="T8" t="s">
-        <v>345</v>
+        <v>346</v>
       </c>
       <c r="X8" t="s">
-        <v>346</v>
+        <v>347</v>
       </c>
       <c r="AA8" t="s">
-        <v>347</v>
+        <v>348</v>
       </c>
       <c r="AB8" t="s">
-        <v>348</v>
+        <v>349</v>
       </c>
       <c r="AE8" t="s">
-        <v>222</v>
+        <v>223</v>
       </c>
       <c r="AF8" t="s">
-        <v>349</v>
+        <v>350</v>
       </c>
       <c r="AH8" t="s">
-        <v>350</v>
+        <v>351</v>
       </c>
       <c r="AI8" t="s">
-        <v>351</v>
+        <v>352</v>
       </c>
       <c r="AJ8" t="s">
-        <v>352</v>
+        <v>353</v>
       </c>
       <c r="AN8" t="s">
-        <v>353</v>
+        <v>354</v>
       </c>
       <c r="AO8" t="s">
-        <v>354</v>
+        <v>355</v>
       </c>
       <c r="AQ8" t="s">
-        <v>355</v>
+        <v>356</v>
       </c>
       <c r="AR8" t="s">
-        <v>356</v>
+        <v>357</v>
       </c>
       <c r="AU8" t="s">
-        <v>222</v>
+        <v>223</v>
       </c>
       <c r="AV8" t="s">
-        <v>357</v>
+        <v>358</v>
       </c>
       <c r="AW8" t="s">
-        <v>358</v>
+        <v>359</v>
       </c>
       <c r="AX8" t="s">
-        <v>359</v>
+        <v>360</v>
       </c>
       <c r="AY8" t="s">
-        <v>360</v>
+        <v>361</v>
       </c>
       <c r="AZ8" t="s">
-        <v>361</v>
+        <v>362</v>
       </c>
       <c r="BA8" t="s">
-        <v>362</v>
+        <v>363</v>
       </c>
       <c r="BC8" t="s">
-        <v>363</v>
+        <v>364</v>
       </c>
       <c r="BD8" t="s">
-        <v>364</v>
+        <v>365</v>
       </c>
       <c r="BE8" t="s">
-        <v>365</v>
+        <v>366</v>
       </c>
       <c r="BF8" t="s">
-        <v>366</v>
+        <v>367</v>
       </c>
       <c r="BG8" t="s">
-        <v>367</v>
+        <v>368</v>
       </c>
       <c r="BI8" t="s">
-        <v>368</v>
+        <v>369</v>
       </c>
       <c r="BN8" t="s">
-        <v>369</v>
+        <v>370</v>
       </c>
       <c r="BQ8" t="s">
-        <v>370</v>
+        <v>371</v>
       </c>
     </row>
     <row r="9" ht="15" customHeight="1" spans="1:69" x14ac:dyDescent="0.25">
       <c r="A9" t="s">
-        <v>371</v>
+        <v>372</v>
       </c>
       <c r="E9" t="s">
-        <v>372</v>
+        <v>373</v>
       </c>
       <c r="F9" t="s">
-        <v>373</v>
+        <v>374</v>
       </c>
       <c r="H9" t="s">
-        <v>374</v>
+        <v>375</v>
       </c>
       <c r="O9" t="s">
-        <v>375</v>
+        <v>376</v>
       </c>
       <c r="T9" t="s">
-        <v>376</v>
+        <v>377</v>
       </c>
       <c r="X9" t="s">
-        <v>377</v>
+        <v>378</v>
       </c>
       <c r="AB9" t="s">
-        <v>378</v>
+        <v>379</v>
       </c>
       <c r="AF9" t="s">
-        <v>379</v>
+        <v>380</v>
       </c>
       <c r="AI9" t="s">
-        <v>380</v>
+        <v>381</v>
       </c>
       <c r="AJ9" t="s">
-        <v>381</v>
+        <v>382</v>
       </c>
       <c r="AO9" t="s">
-        <v>382</v>
+        <v>383</v>
       </c>
       <c r="AV9" t="s">
-        <v>383</v>
+        <v>384</v>
       </c>
       <c r="AW9" t="s">
-        <v>384</v>
+        <v>385</v>
       </c>
       <c r="AX9" t="s">
-        <v>385</v>
+        <v>386</v>
       </c>
       <c r="AY9" t="s">
-        <v>386</v>
+        <v>387</v>
       </c>
       <c r="AZ9" t="s">
-        <v>387</v>
+        <v>388</v>
       </c>
       <c r="BA9" t="s">
-        <v>388</v>
+        <v>389</v>
       </c>
       <c r="BC9" t="s">
-        <v>389</v>
+        <v>390</v>
       </c>
       <c r="BD9" t="s">
-        <v>390</v>
+        <v>391</v>
       </c>
       <c r="BE9" t="s">
-        <v>391</v>
+        <v>392</v>
       </c>
       <c r="BF9" t="s">
-        <v>392</v>
+        <v>393</v>
       </c>
       <c r="BG9" t="s">
-        <v>393</v>
+        <v>394</v>
       </c>
       <c r="BN9" t="s">
-        <v>394</v>
+        <v>395</v>
       </c>
       <c r="BQ9" t="s">
-        <v>395</v>
+        <v>396</v>
       </c>
     </row>
     <row r="10" ht="15" customHeight="1" spans="41:69" x14ac:dyDescent="0.25">
       <c r="AO10" t="s">
-        <v>396</v>
+        <v>397</v>
       </c>
       <c r="AW10" t="s">
-        <v>397</v>
+        <v>398</v>
       </c>
     </row>
     <row r="11" ht="15" customHeight="1" x14ac:dyDescent="0.25"/>

</xml_diff>

<commit_message>
ahl in ice 16.9.
</commit_message>
<xml_diff>
--- a/data/ICEHLdelegacije.xlsx
+++ b/data/ICEHLdelegacije.xlsx
@@ -16,20 +16,20 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="400" uniqueCount="92">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="619" uniqueCount="121">
   <si>
     <t>SternatCh</t>
   </si>
   <si>
+    <t>NikolicMa</t>
+  </si>
+  <si>
     <t>SmetanaLa</t>
   </si>
   <si>
     <t>OfnerCh</t>
   </si>
   <si>
-    <t>NikolicMa</t>
-  </si>
-  <si>
     <t>DurmisOt</t>
   </si>
   <si>
@@ -39,78 +39,87 @@
     <t>PiragicTr</t>
   </si>
   <si>
+    <t>PuffWo</t>
+  </si>
+  <si>
+    <t>JedlickaPe</t>
+  </si>
+  <si>
     <t>SeewaldEl</t>
   </si>
   <si>
     <t>ZrnicMi</t>
   </si>
   <si>
+    <t>BedynekSe</t>
+  </si>
+  <si>
+    <t>HronskyTo</t>
+  </si>
+  <si>
+    <t>ZgoncGa</t>
+  </si>
+  <si>
+    <t>HribarMa</t>
+  </si>
+  <si>
+    <t>KainbergerJu</t>
+  </si>
+  <si>
+    <t>HolzerTo</t>
+  </si>
+  <si>
+    <t>Gatol-schafranekMa</t>
+  </si>
+  <si>
+    <t>VoicanCh</t>
+  </si>
+  <si>
     <t>BärnthalerCh</t>
   </si>
   <si>
-    <t>BedynekSe</t>
-  </si>
-  <si>
-    <t>PuffWo</t>
+    <t>RieckenSi</t>
+  </si>
+  <si>
+    <t>NikolicKr</t>
+  </si>
+  <si>
+    <t>GroznikBo</t>
+  </si>
+  <si>
+    <t>MartinFl</t>
+  </si>
+  <si>
+    <t>WeissAl</t>
+  </si>
+  <si>
+    <t>FichtnerPa</t>
+  </si>
+  <si>
+    <t>SeewaldJe</t>
+  </si>
+  <si>
+    <t>HlavatyAl</t>
+  </si>
+  <si>
+    <t>MantovaniDa</t>
   </si>
   <si>
     <t>RezekGr</t>
   </si>
   <si>
-    <t>RieckenSi</t>
-  </si>
-  <si>
-    <t>HronskyTo</t>
-  </si>
-  <si>
-    <t>JedlickaPe</t>
-  </si>
-  <si>
     <t>SoosDa</t>
   </si>
   <si>
-    <t>ZgoncGa</t>
-  </si>
-  <si>
-    <t>NikolicKr</t>
-  </si>
-  <si>
     <t>FleischmannLu</t>
   </si>
   <si>
-    <t>HribarMa</t>
-  </si>
-  <si>
-    <t>KainbergerJu</t>
-  </si>
-  <si>
     <t>NagyAt</t>
   </si>
   <si>
-    <t>GroznikBo</t>
-  </si>
-  <si>
     <t>SchauerJa</t>
   </si>
   <si>
-    <t>MartinFl</t>
-  </si>
-  <si>
-    <t>HolzerTo</t>
-  </si>
-  <si>
-    <t>WeissAl</t>
-  </si>
-  <si>
-    <t>FichtnerPa</t>
-  </si>
-  <si>
-    <t>Gatol-schafranekMa</t>
-  </si>
-  <si>
-    <t>SeewaldJe</t>
-  </si>
-  <si>
     <t>MuzsikNo</t>
   </si>
   <si>
@@ -120,64 +129,58 @@
     <t>PardatscherUl</t>
   </si>
   <si>
-    <t>HlavatyAl</t>
+    <t>RigoniDa</t>
+  </si>
+  <si>
+    <t>JeramFi</t>
+  </si>
+  <si>
+    <t>NotheggerDa</t>
+  </si>
+  <si>
+    <t>Huber aAn</t>
+  </si>
+  <si>
+    <t>SparerDa</t>
+  </si>
+  <si>
+    <t>WimmlerAl</t>
   </si>
   <si>
     <t>MoidlMa</t>
   </si>
   <si>
-    <t>MantovaniDa</t>
-  </si>
-  <si>
-    <t>SparerDa</t>
-  </si>
-  <si>
-    <t>RigoniDa</t>
-  </si>
-  <si>
-    <t>JeramFi</t>
-  </si>
-  <si>
-    <t>VoicanCh</t>
-  </si>
-  <si>
-    <t>WimmlerAl</t>
-  </si>
-  <si>
     <t>ZacherlPa</t>
   </si>
   <si>
-    <t>NotheggerDa</t>
-  </si>
-  <si>
-    <t>Huber aAn</t>
-  </si>
-  <si>
-    <t>LinesmanZw</t>
-  </si>
-  <si>
     <t>2025-09-12</t>
   </si>
   <si>
     <t>2025-09-14</t>
   </si>
   <si>
+    <t>2025-09-19</t>
+  </si>
+  <si>
     <t>zbrisano</t>
   </si>
   <si>
-    <t>2025-09-19</t>
-  </si>
-  <si>
     <t>2025-09-21</t>
   </si>
   <si>
+    <t>2025-10-12</t>
+  </si>
+  <si>
+    <t>2025-09-28</t>
+  </si>
+  <si>
+    <t>2025-09-27</t>
+  </si>
+  <si>
     <t>2025-09-26</t>
   </si>
   <si>
-    <t>2025-09-27</t>
-  </si>
-  <si>
-    <t>2025-09-28</t>
+    <t>2025-10-03</t>
   </si>
   <si>
     <t>2025-09-20</t>
@@ -186,6 +189,18 @@
     <t>2025-09-23</t>
   </si>
   <si>
+    <t>2025-10-10</t>
+  </si>
+  <si>
+    <t>2025-10-05</t>
+  </si>
+  <si>
+    <t>2025-10-04</t>
+  </si>
+  <si>
+    <t>2025-10-11</t>
+  </si>
+  <si>
     <t>FTC-Telekom Rink;HronskyTo;SmetanaLa;JedlickaPe;MuzsikNo</t>
   </si>
   <si>
@@ -213,6 +228,24 @@
     <t>Merkur Eisstadion Graz;NikolicMa;VoicanCh;BärnthalerCh;Gatol-schafranekMa</t>
   </si>
   <si>
+    <t>Stadthalle Villach;HlavatyAl;KainbergerJu;JeramFi;WimmlerAl</t>
+  </si>
+  <si>
+    <t>Eishalle Wien-Kagran;PiragicTr;SmetanaLa;HribarMa;JedlickaPe</t>
+  </si>
+  <si>
+    <t>Eishalle Feldkirch;HolzerTo;NikolicMa;MartinFl;SparerDa</t>
+  </si>
+  <si>
+    <t>Merkur Eisstadion Graz;HlavatyAl;HronskyTo;DurmisOt;VacziDa</t>
+  </si>
+  <si>
+    <t>Stadthalle Villach;KainbergerJu;ZrnicMi;BedynekSe;ZgoncGa</t>
+  </si>
+  <si>
+    <t>FTC-Telekom Rink;HlavatyAl;SmetanaLa;Gatol-schafranekMa;JedlickaPe</t>
+  </si>
+  <si>
     <t>Hala Tivoli;SoosDa;SternatCh;VacziDa;ZgoncGa</t>
   </si>
   <si>
@@ -234,6 +267,24 @@
     <t>Eisarena Salzburg;SeewaldEl;SmetanaLa;MoidlMa;SeewaldJe</t>
   </si>
   <si>
+    <t>Eishalle Wien-Kagran;OfnerCh;SoosDa;Gatol-schafranekMa;JedlickaPe</t>
+  </si>
+  <si>
+    <t>Tiroler Wasserkraft Arena;HolzerTo;NikolicKr;FleischmannLu;MartinFl</t>
+  </si>
+  <si>
+    <t>Heidi Horten Arena Klagenfurt;RezekGr;SeewaldEl;JeramFi;ZgoncGa</t>
+  </si>
+  <si>
+    <t>Eisarena Salzburg;PiragicTr;SternatCh;JedlickaPe;KoncDa</t>
+  </si>
+  <si>
+    <t>Gabor Ocskay Eisarena;OfnerCh;SeewaldEl;KoncDa;PuffWo</t>
+  </si>
+  <si>
+    <t>Gabor Ocskay Eisarena;OfnerCh;SeewaldEl;MuzsikNo;PuffWo</t>
+  </si>
+  <si>
     <t>Tiroler Wasserkraft Arena;NikolicKr;NikolicMa;FleischmannLu;PardatscherUl</t>
   </si>
   <si>
@@ -252,6 +303,18 @@
     <t>Sparkasse Arena Bozen;NikolicMa;SternatCh;FleischmannLu;WeissAl</t>
   </si>
   <si>
+    <t>Eisarena Salzburg;Huber aAn;NikolicMa;NotheggerDa;SeewaldJe</t>
+  </si>
+  <si>
+    <t>Linz AG Eisarena;FichtnerPa;HronskyTo;DurmisOt;KoncDa</t>
+  </si>
+  <si>
+    <t>Hala Tivoli;SmetanaLa;VoicanCh;HribarMa;RieckenSi</t>
+  </si>
+  <si>
+    <t>Sparkasse Arena Bozen;Huber aAn;NikolicMa;PardatscherUl;RigoniDa</t>
+  </si>
+  <si>
     <t>Heidi Horten Arena Klagenfurt;HlavatyAl;ZrnicMi;BärnthalerCh;HribarMa</t>
   </si>
   <si>
@@ -270,6 +333,18 @@
     <t>Hala Tivoli;PiragicTr;RezekGr;Gatol-schafranekMa;RieckenSi</t>
   </si>
   <si>
+    <t>Gabor Ocskay Eisarena;NagyAt;SternatCh;MuzsikNo;PuffWo</t>
+  </si>
+  <si>
+    <t>Sparkasse Arena Bozen;KainbergerJu;NikolicKr;MantovaniDa;RigoniDa</t>
+  </si>
+  <si>
+    <t>Eishalle Bruneck;GroznikBo;SchauerJa;MantovaniDa;PardatscherUl</t>
+  </si>
+  <si>
+    <t>Eishalle Wien-Kagran;FichtnerPa;HronskyTo;VacziDa;ZacherlPa</t>
+  </si>
+  <si>
     <t>Linz AG Eisarena;KainbergerJu;NagyAt;BedynekSe;Gatol-schafranekMa</t>
   </si>
   <si>
@@ -285,6 +360,15 @@
     <t>Sparkasse Arena Bozen;NikolicKr;SchauerJa;PardatscherUl;RigoniDa</t>
   </si>
   <si>
+    <t>Linz AG Eisarena;VoicanCh;ZrnicMi;WeissAl;ZgoncGa</t>
+  </si>
+  <si>
+    <t>Stadthalle Villach;GroznikBo;Huber aAn;NotheggerDa;SeewaldJe</t>
+  </si>
+  <si>
+    <t>Heidi Horten Arena Klagenfurt;HolzerTo;SternatCh;DurmisOt;WeissAl</t>
+  </si>
+  <si>
     <t>Sparkasse Arena Bozen;GroznikBo;OfnerCh;MantovaniDa;PuffWo</t>
   </si>
   <si>
@@ -292,13 +376,16 @@
   </si>
   <si>
     <t>Hala Tivoli;NagyAt;OfnerCh;MuzsikNo;PuffWo</t>
+  </si>
+  <si>
+    <t>Hala Tivoli;PiragicTr;VoicanCh;BärnthalerCh;RieckenSi</t>
   </si>
 </sst>
 </file>
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:x16r2="http://schemas.microsoft.com/office/spreadsheetml/2015/02/main" mc:Ignorable="x14ac x16r2">
-  <fonts count="1" x14ac:knownFonts="1">
+  <fonts count="2" x14ac:knownFonts="1">
     <font>
       <color theme="1"/>
       <family val="2"/>
@@ -306,13 +393,26 @@
       <sz val="11"/>
       <name val="Calibri"/>
     </font>
+    <font>
+      <charset val="238"/>
+      <color rgb="FF006100"/>
+      <family val="2"/>
+      <scheme val="minor"/>
+      <sz val="11"/>
+      <name val="Calibri"/>
+    </font>
   </fonts>
-  <fills count="2">
+  <fills count="3">
     <fill>
       <patternFill patternType="none"/>
     </fill>
     <fill>
       <patternFill patternType="gray125"/>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor rgb="FFC6EFCE"/>
+      </patternFill>
     </fill>
   </fills>
   <borders count="1">
@@ -327,8 +427,9 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="1">
+  <cellXfs count="2">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
+    <xf numFmtId="0" fontId="1" fillId="2" borderId="0" xfId="0" applyFont="1" applyFill="1"/>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0"/>
@@ -609,7 +710,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" mc:Ignorable="x14ac">
-  <dimension ref="A2:AU134"/>
+  <dimension ref="A2:AT134"/>
   <sheetFormatPr defaultRowHeight="14.45" outlineLevelRow="0" outlineLevelCol="0" x14ac:dyDescent="0.25" customHeight="1"/>
   <cols>
     <col min="1" max="1" width="12.28515625" customWidth="1"/>
@@ -667,193 +768,189 @@
     <col min="53" max="53" width="10.140625" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="2" ht="14.45" customHeight="1" spans="1:46" x14ac:dyDescent="0.25">
+    <row r="2" ht="14.45" customHeight="1" spans="1:45" x14ac:dyDescent="0.25">
       <c r="A2">
         <f>COUNTIF(A4:A118,"&lt;&gt;")</f>
-        <v>7</v>
+        <v>10</v>
       </c>
       <c r="B2">
-        <f>COUNTIF(B4:B118,"&lt;&gt;")</f>
-        <v>6</v>
+        <f>COUNTIF(B4:B117,"&lt;&gt;")</f>
+        <v>10</v>
       </c>
       <c r="C2">
         <f>COUNTIF(C4:C118,"&lt;&gt;")</f>
-        <v>6</v>
+        <v>9</v>
       </c>
       <c r="D2">
         <f>COUNTIF(D4:D118,"&lt;&gt;")</f>
-        <v>6</v>
+        <v>9</v>
       </c>
       <c r="E2">
         <f>COUNTIF(E4:E118,"&lt;&gt;")</f>
-        <v>5</v>
+        <v>8</v>
       </c>
       <c r="F2">
         <f>COUNTIF(F4:F118,"&lt;&gt;")</f>
-        <v>5</v>
+        <v>8</v>
       </c>
       <c r="G2">
         <f>COUNTIF(G4:G118,"&lt;&gt;")</f>
-        <v>5</v>
+        <v>8</v>
       </c>
       <c r="H2">
         <f>COUNTIF(H4:H118,"&lt;&gt;")</f>
-        <v>4</v>
+        <v>7</v>
       </c>
       <c r="I2">
         <f>COUNTIF(I4:I118,"&lt;&gt;")</f>
-        <v>4</v>
+        <v>7</v>
       </c>
       <c r="J2">
-        <f>COUNTIF(J4:J118,"&lt;&gt;")</f>
-        <v>4</v>
+        <f>COUNTIF(J4:J117,"&lt;&gt;")</f>
+        <v>6</v>
       </c>
       <c r="K2">
         <f>COUNTIF(K4:K118,"&lt;&gt;")</f>
-        <v>4</v>
+        <v>6</v>
       </c>
       <c r="L2">
         <f>COUNTIF(L4:L118,"&lt;&gt;")</f>
-        <v>4</v>
+        <v>6</v>
       </c>
       <c r="M2">
-        <f>COUNTIF(M4:M117,"&lt;&gt;")</f>
-        <v>3</v>
+        <f>COUNTIF(M4:M118,"&lt;&gt;")</f>
+        <v>6</v>
       </c>
       <c r="N2">
         <f>COUNTIF(N4:N118,"&lt;&gt;")</f>
-        <v>4</v>
+        <v>6</v>
       </c>
       <c r="O2">
         <f>COUNTIF(O4:O118,"&lt;&gt;")</f>
-        <v>3</v>
+        <v>6</v>
       </c>
       <c r="P2">
         <f>COUNTIF(P4:P118,"&lt;&gt;")</f>
-        <v>3</v>
+        <v>6</v>
       </c>
       <c r="Q2">
         <f>COUNTIF(Q4:Q118,"&lt;&gt;")</f>
-        <v>3</v>
+        <v>6</v>
       </c>
       <c r="R2">
-        <f>COUNTIF(R4:R118,"&lt;&gt;")</f>
-        <v>3</v>
+        <f>COUNTIF(R4:R117,"&lt;&gt;")</f>
+        <v>6</v>
       </c>
       <c r="S2">
         <f>COUNTIF(S4:S118,"&lt;&gt;")</f>
-        <v>3</v>
+        <v>6</v>
       </c>
       <c r="T2">
-        <f>COUNTIF(T4:T118,"&lt;&gt;")</f>
-        <v>3</v>
+        <f>COUNTIF(T4:T117,"&lt;&gt;")</f>
+        <v>5</v>
       </c>
       <c r="U2">
-        <f>COUNTIF(U4:U118,"&lt;&gt;")</f>
-        <v>3</v>
+        <f>COUNTIF(U4:U117,"&lt;&gt;")</f>
+        <v>5</v>
       </c>
       <c r="V2">
         <f>COUNTIF(V4:V118,"&lt;&gt;")</f>
-        <v>3</v>
+        <v>5</v>
       </c>
       <c r="W2">
         <f>COUNTIF(W4:W118,"&lt;&gt;")</f>
-        <v>3</v>
+        <v>5</v>
       </c>
       <c r="X2">
         <f>COUNTIF(X4:X118,"&lt;&gt;")</f>
-        <v>3</v>
+        <v>5</v>
       </c>
       <c r="Y2">
         <f>COUNTIF(Y4:Y118,"&lt;&gt;")</f>
-        <v>3</v>
+        <v>5</v>
       </c>
       <c r="Z2">
         <f>COUNTIF(Z4:Z118,"&lt;&gt;")</f>
-        <v>3</v>
+        <v>5</v>
       </c>
       <c r="AA2">
         <f>COUNTIF(AA4:AA118,"&lt;&gt;")</f>
-        <v>3</v>
+        <v>5</v>
       </c>
       <c r="AB2">
         <f>COUNTIF(AB4:AB118,"&lt;&gt;")</f>
-        <v>3</v>
+        <v>5</v>
       </c>
       <c r="AC2">
         <f>COUNTIF(AC4:AC118,"&lt;&gt;")</f>
-        <v>3</v>
+        <v>5</v>
       </c>
       <c r="AD2">
-        <f>COUNTIF(AD4:AD118,"&lt;&gt;")</f>
-        <v>3</v>
+        <f>COUNTIF(AD4:AD117,"&lt;&gt;")</f>
+        <v>4</v>
       </c>
       <c r="AE2">
         <f>COUNTIF(AE4:AE118,"&lt;&gt;")</f>
-        <v>3</v>
+        <v>4</v>
       </c>
       <c r="AF2">
         <f>COUNTIF(AF4:AF118,"&lt;&gt;")</f>
-        <v>2</v>
+        <v>4</v>
       </c>
       <c r="AG2">
         <f>COUNTIF(AG4:AG118,"&lt;&gt;")</f>
-        <v>2</v>
+        <v>4</v>
       </c>
       <c r="AH2">
         <f>COUNTIF(AH4:AH118,"&lt;&gt;")</f>
-        <v>2</v>
+        <v>4</v>
       </c>
       <c r="AI2">
         <f>COUNTIF(AI4:AI118,"&lt;&gt;")</f>
-        <v>2</v>
+        <v>4</v>
       </c>
       <c r="AJ2">
         <f>COUNTIF(AJ4:AJ118,"&lt;&gt;")</f>
-        <v>2</v>
+        <v>4</v>
       </c>
       <c r="AK2">
         <f>COUNTIF(AK4:AK118,"&lt;&gt;")</f>
-        <v>2</v>
+        <v>4</v>
       </c>
       <c r="AL2">
         <f>COUNTIF(AL4:AL118,"&lt;&gt;")</f>
-        <v>2</v>
+        <v>4</v>
       </c>
       <c r="AM2">
         <f>COUNTIF(AM4:AM118,"&lt;&gt;")</f>
-        <v>2</v>
+        <v>4</v>
       </c>
       <c r="AN2">
         <f>COUNTIF(AN4:AN118,"&lt;&gt;")</f>
-        <v>2</v>
+        <v>4</v>
       </c>
       <c r="AO2">
         <f>COUNTIF(AO4:AO118,"&lt;&gt;")</f>
-        <v>2</v>
+        <v>4</v>
       </c>
       <c r="AP2">
         <f>COUNTIF(AP4:AP118,"&lt;&gt;")</f>
-        <v>2</v>
+        <v>3</v>
       </c>
       <c r="AQ2">
         <f>COUNTIF(AQ4:AQ118,"&lt;&gt;")</f>
-        <v>2</v>
+        <v>3</v>
       </c>
       <c r="AR2">
         <f>COUNTIF(AR4:AR118,"&lt;&gt;")</f>
         <v>2</v>
       </c>
       <c r="AS2">
-        <f>COUNTIF(AS4:AS118,"&lt;&gt;")</f>
+        <f>COUNTIF(AS4:AS116,"&lt;&gt;")</f>
         <v>1</v>
       </c>
-      <c r="AT2">
-        <f>COUNTIF(AT4:AT118,"&lt;&gt;")</f>
-        <v>1</v>
-      </c>
     </row>
-    <row r="3" ht="15" customHeight="1" spans="1:47" x14ac:dyDescent="0.25">
+    <row r="3" ht="15" customHeight="1" spans="1:46" x14ac:dyDescent="0.25">
       <c r="A3" t="s">
         <v>0</v>
       </c>
@@ -872,7 +969,7 @@
       <c r="F3" t="s">
         <v>5</v>
       </c>
-      <c r="G3" t="s">
+      <c r="G3" s="1" t="s">
         <v>6</v>
       </c>
       <c r="H3" t="s">
@@ -884,7 +981,7 @@
       <c r="J3" t="s">
         <v>9</v>
       </c>
-      <c r="K3" t="s">
+      <c r="K3" s="1" t="s">
         <v>10</v>
       </c>
       <c r="L3" t="s">
@@ -893,10 +990,10 @@
       <c r="M3" t="s">
         <v>12</v>
       </c>
-      <c r="N3" t="s">
+      <c r="N3" s="1" t="s">
         <v>13</v>
       </c>
-      <c r="O3" t="s">
+      <c r="O3" s="1" t="s">
         <v>14</v>
       </c>
       <c r="P3" t="s">
@@ -920,7 +1017,7 @@
       <c r="V3" t="s">
         <v>21</v>
       </c>
-      <c r="W3" t="s">
+      <c r="W3" s="1" t="s">
         <v>22</v>
       </c>
       <c r="X3" t="s">
@@ -941,7 +1038,7 @@
       <c r="AC3" t="s">
         <v>28</v>
       </c>
-      <c r="AD3" t="s">
+      <c r="AD3" s="1" t="s">
         <v>29</v>
       </c>
       <c r="AE3" t="s">
@@ -968,7 +1065,7 @@
       <c r="AL3" t="s">
         <v>37</v>
       </c>
-      <c r="AM3" t="s">
+      <c r="AM3" s="1" t="s">
         <v>38</v>
       </c>
       <c r="AN3" t="s">
@@ -989,58 +1086,55 @@
       <c r="AS3" t="s">
         <v>44</v>
       </c>
-      <c r="AT3" t="s">
+    </row>
+    <row r="4" ht="15" customHeight="1" spans="1:45" x14ac:dyDescent="0.25">
+      <c r="A4" t="s">
         <v>45</v>
-      </c>
-    </row>
-    <row r="4" ht="15" customHeight="1" spans="1:46" x14ac:dyDescent="0.25">
-      <c r="A4" t="s">
-        <v>46</v>
       </c>
       <c r="B4" t="s">
         <v>46</v>
       </c>
       <c r="C4" t="s">
+        <v>45</v>
+      </c>
+      <c r="D4" t="s">
+        <v>45</v>
+      </c>
+      <c r="E4" t="s">
         <v>46</v>
       </c>
-      <c r="D4" t="s">
+      <c r="F4" t="s">
+        <v>46</v>
+      </c>
+      <c r="G4" t="s">
+        <v>46</v>
+      </c>
+      <c r="H4" t="s">
+        <v>45</v>
+      </c>
+      <c r="I4" t="s">
+        <v>45</v>
+      </c>
+      <c r="J4" t="s">
         <v>47</v>
       </c>
-      <c r="E4" t="s">
-        <v>47</v>
-      </c>
-      <c r="F4" t="s">
-        <v>47</v>
-      </c>
-      <c r="G4" t="s">
-        <v>47</v>
-      </c>
-      <c r="H4" t="s">
-        <v>48</v>
-      </c>
-      <c r="I4" t="s">
-        <v>46</v>
-      </c>
-      <c r="J4" t="s">
-        <v>46</v>
-      </c>
       <c r="K4" t="s">
-        <v>46</v>
+        <v>45</v>
       </c>
       <c r="L4" t="s">
-        <v>46</v>
+        <v>45</v>
       </c>
       <c r="M4" t="s">
-        <v>47</v>
+        <v>45</v>
       </c>
       <c r="N4" t="s">
-        <v>47</v>
+        <v>45</v>
       </c>
       <c r="O4" t="s">
-        <v>46</v>
+        <v>45</v>
       </c>
       <c r="P4" t="s">
-        <v>46</v>
+        <v>45</v>
       </c>
       <c r="Q4" t="s">
         <v>46</v>
@@ -1049,67 +1143,67 @@
         <v>46</v>
       </c>
       <c r="S4" t="s">
-        <v>46</v>
+        <v>47</v>
       </c>
       <c r="T4" t="s">
-        <v>46</v>
+        <v>45</v>
       </c>
       <c r="U4" t="s">
         <v>46</v>
       </c>
       <c r="V4" t="s">
-        <v>46</v>
+        <v>45</v>
       </c>
       <c r="W4" t="s">
-        <v>46</v>
+        <v>45</v>
       </c>
       <c r="X4" t="s">
         <v>46</v>
       </c>
       <c r="Y4" t="s">
-        <v>47</v>
+        <v>46</v>
       </c>
       <c r="Z4" t="s">
-        <v>47</v>
+        <v>46</v>
       </c>
       <c r="AA4" t="s">
-        <v>47</v>
+        <v>48</v>
       </c>
       <c r="AB4" t="s">
-        <v>47</v>
+        <v>45</v>
       </c>
       <c r="AC4" t="s">
-        <v>47</v>
+        <v>45</v>
       </c>
       <c r="AD4" t="s">
-        <v>47</v>
+        <v>46</v>
       </c>
       <c r="AE4" t="s">
-        <v>48</v>
+        <v>45</v>
       </c>
       <c r="AF4" t="s">
-        <v>46</v>
+        <v>45</v>
       </c>
       <c r="AG4" t="s">
-        <v>46</v>
+        <v>45</v>
       </c>
       <c r="AH4" t="s">
         <v>46</v>
       </c>
       <c r="AI4" t="s">
+        <v>45</v>
+      </c>
+      <c r="AJ4" t="s">
+        <v>45</v>
+      </c>
+      <c r="AK4" t="s">
+        <v>45</v>
+      </c>
+      <c r="AL4" t="s">
         <v>46</v>
       </c>
-      <c r="AJ4" t="s">
-        <v>48</v>
-      </c>
-      <c r="AK4" t="s">
+      <c r="AM4" t="s">
         <v>46</v>
-      </c>
-      <c r="AL4" t="s">
-        <v>47</v>
-      </c>
-      <c r="AM4" t="s">
-        <v>47</v>
       </c>
       <c r="AN4" t="s">
         <v>47</v>
@@ -1118,45 +1212,42 @@
         <v>49</v>
       </c>
       <c r="AP4" t="s">
-        <v>49</v>
+        <v>46</v>
       </c>
       <c r="AQ4" t="s">
+        <v>47</v>
+      </c>
+      <c r="AR4" t="s">
         <v>48</v>
-      </c>
-      <c r="AR4" t="s">
-        <v>49</v>
       </c>
       <c r="AS4" t="s">
         <v>50</v>
       </c>
-      <c r="AT4" t="s">
-        <v>48</v>
-      </c>
     </row>
-    <row r="5" ht="15" customHeight="1" spans="1:46" x14ac:dyDescent="0.25">
+    <row r="5" ht="15" customHeight="1" spans="1:45" x14ac:dyDescent="0.25">
       <c r="A5" t="s">
-        <v>47</v>
+        <v>46</v>
       </c>
       <c r="B5" t="s">
         <v>47</v>
       </c>
       <c r="C5" t="s">
+        <v>46</v>
+      </c>
+      <c r="D5" t="s">
+        <v>46</v>
+      </c>
+      <c r="E5" t="s">
         <v>47</v>
       </c>
-      <c r="D5" t="s">
-        <v>49</v>
-      </c>
-      <c r="E5" t="s">
-        <v>49</v>
-      </c>
       <c r="F5" t="s">
-        <v>49</v>
+        <v>47</v>
       </c>
       <c r="G5" t="s">
-        <v>49</v>
+        <v>47</v>
       </c>
       <c r="H5" t="s">
-        <v>49</v>
+        <v>46</v>
       </c>
       <c r="I5" t="s">
         <v>47</v>
@@ -1165,230 +1256,260 @@
         <v>49</v>
       </c>
       <c r="K5" t="s">
+        <v>46</v>
+      </c>
+      <c r="L5" t="s">
+        <v>46</v>
+      </c>
+      <c r="M5" t="s">
         <v>47</v>
       </c>
-      <c r="L5" t="s">
+      <c r="N5" t="s">
         <v>47</v>
       </c>
-      <c r="M5" t="s">
-        <v>50</v>
-      </c>
-      <c r="N5" t="s">
-        <v>49</v>
-      </c>
       <c r="O5" t="s">
-        <v>49</v>
+        <v>46</v>
       </c>
       <c r="P5" t="s">
-        <v>49</v>
+        <v>47</v>
       </c>
       <c r="Q5" t="s">
+        <v>47</v>
+      </c>
+      <c r="R5" t="s">
         <v>51</v>
       </c>
-      <c r="R5" t="s">
-        <v>49</v>
-      </c>
       <c r="S5" t="s">
+        <v>48</v>
+      </c>
+      <c r="T5" t="s">
         <v>47</v>
-      </c>
-      <c r="T5" t="s">
-        <v>51</v>
       </c>
       <c r="U5" t="s">
         <v>47</v>
       </c>
       <c r="V5" t="s">
-        <v>49</v>
+        <v>46</v>
       </c>
       <c r="W5" t="s">
-        <v>50</v>
+        <v>46</v>
       </c>
       <c r="X5" t="s">
         <v>47</v>
       </c>
       <c r="Y5" t="s">
-        <v>50</v>
+        <v>52</v>
       </c>
       <c r="Z5" t="s">
         <v>49</v>
       </c>
       <c r="AA5" t="s">
+        <v>53</v>
+      </c>
+      <c r="AB5" t="s">
+        <v>53</v>
+      </c>
+      <c r="AC5" t="s">
         <v>49</v>
       </c>
-      <c r="AB5" t="s">
+      <c r="AD5" t="s">
+        <v>49</v>
+      </c>
+      <c r="AE5" t="s">
+        <v>53</v>
+      </c>
+      <c r="AF5" t="s">
+        <v>53</v>
+      </c>
+      <c r="AG5" t="s">
+        <v>49</v>
+      </c>
+      <c r="AH5" t="s">
+        <v>49</v>
+      </c>
+      <c r="AI5" t="s">
+        <v>49</v>
+      </c>
+      <c r="AJ5" t="s">
+        <v>49</v>
+      </c>
+      <c r="AK5" t="s">
+        <v>53</v>
+      </c>
+      <c r="AL5" t="s">
+        <v>53</v>
+      </c>
+      <c r="AM5" t="s">
+        <v>49</v>
+      </c>
+      <c r="AN5" t="s">
+        <v>49</v>
+      </c>
+      <c r="AO5" t="s">
+        <v>54</v>
+      </c>
+      <c r="AP5" t="s">
         <v>52</v>
       </c>
-      <c r="AC5" t="s">
-        <v>50</v>
-      </c>
-      <c r="AD5" t="s">
-        <v>48</v>
-      </c>
-      <c r="AE5" t="s">
+      <c r="AQ5" t="s">
+        <v>53</v>
+      </c>
+      <c r="AR5" t="s">
         <v>51</v>
-      </c>
-      <c r="AF5" t="s">
-        <v>50</v>
-      </c>
-      <c r="AG5" t="s">
-        <v>50</v>
-      </c>
-      <c r="AH5" t="s">
-        <v>51</v>
-      </c>
-      <c r="AI5" t="s">
-        <v>51</v>
-      </c>
-      <c r="AJ5" t="s">
-        <v>53</v>
-      </c>
-      <c r="AK5" t="s">
-        <v>50</v>
-      </c>
-      <c r="AL5" t="s">
-        <v>52</v>
-      </c>
-      <c r="AM5" t="s">
-        <v>51</v>
-      </c>
-      <c r="AN5" t="s">
-        <v>50</v>
-      </c>
-      <c r="AO5" t="s">
-        <v>48</v>
-      </c>
-      <c r="AP5" t="s">
-        <v>51</v>
-      </c>
-      <c r="AQ5" t="s">
-        <v>48</v>
-      </c>
-      <c r="AR5" t="s">
-        <v>50</v>
       </c>
     </row>
     <row r="6" ht="15" customHeight="1" spans="1:44" x14ac:dyDescent="0.25">
       <c r="A6" t="s">
+        <v>47</v>
+      </c>
+      <c r="B6" t="s">
+        <v>53</v>
+      </c>
+      <c r="C6" t="s">
+        <v>47</v>
+      </c>
+      <c r="D6" t="s">
+        <v>47</v>
+      </c>
+      <c r="E6" t="s">
+        <v>55</v>
+      </c>
+      <c r="F6" t="s">
+        <v>55</v>
+      </c>
+      <c r="G6" t="s">
+        <v>55</v>
+      </c>
+      <c r="H6" t="s">
         <v>49</v>
-      </c>
-      <c r="B6" t="s">
-        <v>49</v>
-      </c>
-      <c r="C6" t="s">
-        <v>49</v>
-      </c>
-      <c r="D6" t="s">
-        <v>48</v>
-      </c>
-      <c r="E6" t="s">
-        <v>54</v>
-      </c>
-      <c r="F6" t="s">
-        <v>54</v>
-      </c>
-      <c r="G6" t="s">
-        <v>54</v>
-      </c>
-      <c r="H6" t="s">
-        <v>50</v>
       </c>
       <c r="I6" t="s">
         <v>49</v>
       </c>
       <c r="J6" t="s">
-        <v>48</v>
+        <v>51</v>
       </c>
       <c r="K6" t="s">
-        <v>50</v>
+        <v>47</v>
       </c>
       <c r="L6" t="s">
-        <v>50</v>
+        <v>49</v>
       </c>
       <c r="M6" t="s">
+        <v>49</v>
+      </c>
+      <c r="N6" t="s">
+        <v>49</v>
+      </c>
+      <c r="O6" t="s">
+        <v>49</v>
+      </c>
+      <c r="P6" t="s">
         <v>53</v>
       </c>
-      <c r="N6" t="s">
-        <v>48</v>
-      </c>
-      <c r="O6" t="s">
-        <v>50</v>
-      </c>
-      <c r="P6" t="s">
-        <v>50</v>
-      </c>
       <c r="Q6" t="s">
+        <v>52</v>
+      </c>
+      <c r="R6" t="s">
+        <v>56</v>
+      </c>
+      <c r="S6" t="s">
+        <v>56</v>
+      </c>
+      <c r="T6" t="s">
+        <v>51</v>
+      </c>
+      <c r="U6" t="s">
+        <v>51</v>
+      </c>
+      <c r="V6" t="s">
         <v>53</v>
-      </c>
-      <c r="R6" t="s">
-        <v>50</v>
-      </c>
-      <c r="S6" t="s">
-        <v>51</v>
-      </c>
-      <c r="T6" t="s">
-        <v>53</v>
-      </c>
-      <c r="U6" t="s">
-        <v>50</v>
-      </c>
-      <c r="V6" t="s">
-        <v>51</v>
       </c>
       <c r="W6" t="s">
         <v>53</v>
       </c>
       <c r="X6" t="s">
-        <v>51</v>
+        <v>53</v>
       </c>
       <c r="Y6" t="s">
         <v>51</v>
       </c>
       <c r="Z6" t="s">
+        <v>53</v>
+      </c>
+      <c r="AA6" t="s">
         <v>51</v>
       </c>
-      <c r="AA6" t="s">
+      <c r="AB6" t="s">
+        <v>54</v>
+      </c>
+      <c r="AC6" t="s">
+        <v>53</v>
+      </c>
+      <c r="AD6" t="s">
+        <v>51</v>
+      </c>
+      <c r="AE6" t="s">
+        <v>51</v>
+      </c>
+      <c r="AF6" t="s">
+        <v>51</v>
+      </c>
+      <c r="AG6" t="s">
+        <v>51</v>
+      </c>
+      <c r="AH6" t="s">
+        <v>53</v>
+      </c>
+      <c r="AI6" t="s">
+        <v>54</v>
+      </c>
+      <c r="AJ6" t="s">
+        <v>57</v>
+      </c>
+      <c r="AK6" t="s">
+        <v>57</v>
+      </c>
+      <c r="AL6" t="s">
+        <v>58</v>
+      </c>
+      <c r="AM6" t="s">
+        <v>54</v>
+      </c>
+      <c r="AN6" t="s">
+        <v>54</v>
+      </c>
+      <c r="AO6" t="s">
+        <v>58</v>
+      </c>
+      <c r="AP6" t="s">
+        <v>58</v>
+      </c>
+      <c r="AQ6" t="s">
+        <v>54</v>
+      </c>
+    </row>
+    <row r="7" ht="15" customHeight="1" spans="1:43" x14ac:dyDescent="0.25">
+      <c r="A7" t="s">
+        <v>49</v>
+      </c>
+      <c r="B7" t="s">
         <v>52</v>
       </c>
-      <c r="AB6" t="s">
+      <c r="C7" t="s">
+        <v>49</v>
+      </c>
+      <c r="D7" t="s">
+        <v>49</v>
+      </c>
+      <c r="E7" t="s">
         <v>53</v>
       </c>
-      <c r="AC6" t="s">
-        <v>51</v>
-      </c>
-      <c r="AD6" t="s">
+      <c r="F7" t="s">
         <v>53</v>
       </c>
-      <c r="AE6" t="s">
+      <c r="G7" t="s">
         <v>53</v>
-      </c>
-      <c r="AK6" t="s">
-        <v>51</v>
-      </c>
-      <c r="AO6" t="s">
-        <v>55</v>
-      </c>
-    </row>
-    <row r="7" ht="15" customHeight="1" spans="1:41" x14ac:dyDescent="0.25">
-      <c r="A7" t="s">
-        <v>50</v>
-      </c>
-      <c r="B7" t="s">
-        <v>50</v>
-      </c>
-      <c r="C7" t="s">
-        <v>50</v>
-      </c>
-      <c r="D7" t="s">
-        <v>51</v>
-      </c>
-      <c r="E7" t="s">
-        <v>51</v>
-      </c>
-      <c r="F7" t="s">
-        <v>51</v>
-      </c>
-      <c r="G7" t="s">
-        <v>51</v>
       </c>
       <c r="H7" t="s">
         <v>53</v>
@@ -1397,36 +1518,114 @@
         <v>54</v>
       </c>
       <c r="J7" t="s">
-        <v>53</v>
+        <v>58</v>
       </c>
       <c r="K7" t="s">
-        <v>53</v>
+        <v>55</v>
       </c>
       <c r="L7" t="s">
         <v>51</v>
       </c>
+      <c r="M7" t="s">
+        <v>58</v>
+      </c>
       <c r="N7" t="s">
+        <v>54</v>
+      </c>
+      <c r="O7" t="s">
         <v>53</v>
       </c>
+      <c r="P7" t="s">
+        <v>54</v>
+      </c>
+      <c r="Q7" t="s">
+        <v>59</v>
+      </c>
+      <c r="R7" t="s">
+        <v>45</v>
+      </c>
+      <c r="S7" t="s">
+        <v>54</v>
+      </c>
+      <c r="T7" t="s">
+        <v>56</v>
+      </c>
       <c r="U7" t="s">
-        <v>51</v>
+        <v>57</v>
+      </c>
+      <c r="V7" t="s">
+        <v>59</v>
+      </c>
+      <c r="W7" t="s">
+        <v>58</v>
+      </c>
+      <c r="X7" t="s">
+        <v>59</v>
+      </c>
+      <c r="Y7" t="s">
+        <v>54</v>
+      </c>
+      <c r="Z7" t="s">
+        <v>58</v>
+      </c>
+      <c r="AA7" t="s">
+        <v>54</v>
+      </c>
+      <c r="AB7" t="s">
+        <v>57</v>
+      </c>
+      <c r="AC7" t="s">
+        <v>58</v>
       </c>
       <c r="AD7" t="s">
-        <v>55</v>
+        <v>58</v>
+      </c>
+      <c r="AE7" t="s">
+        <v>54</v>
+      </c>
+      <c r="AF7" t="s">
+        <v>59</v>
+      </c>
+      <c r="AG7" t="s">
+        <v>54</v>
+      </c>
+      <c r="AH7" t="s">
+        <v>57</v>
+      </c>
+      <c r="AI7" t="s">
+        <v>50</v>
+      </c>
+      <c r="AJ7" t="s">
+        <v>50</v>
+      </c>
+      <c r="AK7" t="s">
+        <v>50</v>
+      </c>
+      <c r="AL7" t="s">
+        <v>50</v>
+      </c>
+      <c r="AM7" t="s">
+        <v>58</v>
+      </c>
+      <c r="AN7" t="s">
+        <v>58</v>
+      </c>
+      <c r="AO7" t="s">
+        <v>50</v>
       </c>
     </row>
-    <row r="8" ht="15" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
+    <row r="8" ht="15" customHeight="1" spans="1:41" x14ac:dyDescent="0.25">
       <c r="A8" t="s">
-        <v>51</v>
+        <v>53</v>
       </c>
       <c r="B8" t="s">
         <v>51</v>
       </c>
       <c r="C8" t="s">
-        <v>51</v>
+        <v>53</v>
       </c>
       <c r="D8" t="s">
-        <v>52</v>
+        <v>53</v>
       </c>
       <c r="E8" t="s">
         <v>52</v>
@@ -1435,48 +1634,209 @@
         <v>52</v>
       </c>
       <c r="G8" t="s">
+        <v>51</v>
+      </c>
+      <c r="H8" t="s">
+        <v>54</v>
+      </c>
+      <c r="I8" t="s">
+        <v>59</v>
+      </c>
+      <c r="J8" t="s">
+        <v>60</v>
+      </c>
+      <c r="K8" t="s">
+        <v>54</v>
+      </c>
+      <c r="L8" t="s">
         <v>53</v>
       </c>
-      <c r="J8" t="s">
-        <v>55</v>
-      </c>
-      <c r="K8" t="s">
-        <v>51</v>
-      </c>
-      <c r="AD8" t="s">
-        <v>46</v>
+      <c r="M8" t="s">
+        <v>57</v>
+      </c>
+      <c r="N8" t="s">
+        <v>58</v>
+      </c>
+      <c r="O8" t="s">
+        <v>59</v>
+      </c>
+      <c r="P8" t="s">
+        <v>58</v>
+      </c>
+      <c r="Q8" t="s">
+        <v>58</v>
+      </c>
+      <c r="R8" t="s">
+        <v>54</v>
+      </c>
+      <c r="S8" t="s">
+        <v>57</v>
+      </c>
+      <c r="T8" t="s">
+        <v>50</v>
+      </c>
+      <c r="U8" t="s">
+        <v>50</v>
+      </c>
+      <c r="V8" t="s">
+        <v>58</v>
+      </c>
+      <c r="W8" t="s">
+        <v>57</v>
+      </c>
+      <c r="X8" t="s">
+        <v>58</v>
+      </c>
+      <c r="Y8" t="s">
+        <v>50</v>
+      </c>
+      <c r="Z8" t="s">
+        <v>50</v>
+      </c>
+      <c r="AA8" t="s">
+        <v>58</v>
+      </c>
+      <c r="AB8" t="s">
+        <v>50</v>
+      </c>
+      <c r="AC8" t="s">
+        <v>57</v>
       </c>
     </row>
-    <row r="9" ht="15" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
+    <row r="9" ht="15" customHeight="1" spans="1:29" x14ac:dyDescent="0.25">
       <c r="A9" t="s">
         <v>52</v>
       </c>
       <c r="B9" t="s">
-        <v>53</v>
+        <v>56</v>
       </c>
       <c r="C9" t="s">
+        <v>51</v>
+      </c>
+      <c r="D9" t="s">
         <v>52</v>
       </c>
-      <c r="D9" t="s">
-        <v>53</v>
+      <c r="E9" t="s">
+        <v>58</v>
+      </c>
+      <c r="F9" t="s">
+        <v>58</v>
+      </c>
+      <c r="G9" t="s">
+        <v>59</v>
+      </c>
+      <c r="H9" t="s">
+        <v>60</v>
+      </c>
+      <c r="I9" t="s">
+        <v>57</v>
+      </c>
+      <c r="J9" t="s">
+        <v>50</v>
+      </c>
+      <c r="K9" t="s">
+        <v>60</v>
+      </c>
+      <c r="L9" t="s">
+        <v>60</v>
+      </c>
+      <c r="M9" t="s">
+        <v>50</v>
+      </c>
+      <c r="N9" t="s">
+        <v>60</v>
+      </c>
+      <c r="O9" t="s">
+        <v>57</v>
+      </c>
+      <c r="P9" t="s">
+        <v>60</v>
+      </c>
+      <c r="Q9" t="s">
+        <v>50</v>
+      </c>
+      <c r="R9" t="s">
+        <v>50</v>
+      </c>
+      <c r="S9" t="s">
+        <v>50</v>
       </c>
     </row>
-    <row r="10" ht="15" customHeight="1" spans="1:4" x14ac:dyDescent="0.25">
+    <row r="10" ht="15" customHeight="1" spans="1:19" x14ac:dyDescent="0.25">
       <c r="A10" t="s">
-        <v>53</v>
+        <v>51</v>
+      </c>
+      <c r="B10" t="s">
+        <v>45</v>
+      </c>
+      <c r="C10" t="s">
+        <v>59</v>
       </c>
       <c r="D10" t="s">
-        <v>55</v>
+        <v>54</v>
+      </c>
+      <c r="E10" t="s">
+        <v>57</v>
+      </c>
+      <c r="F10" t="s">
+        <v>57</v>
+      </c>
+      <c r="G10" t="s">
+        <v>57</v>
+      </c>
+      <c r="H10" t="s">
+        <v>50</v>
+      </c>
+      <c r="I10" t="s">
+        <v>50</v>
       </c>
     </row>
-    <row r="11" ht="15" customHeight="1" spans="1:4" x14ac:dyDescent="0.25">
+    <row r="11" ht="15" customHeight="1" spans="1:9" x14ac:dyDescent="0.25">
+      <c r="A11" t="s">
+        <v>54</v>
+      </c>
+      <c r="B11" t="s">
+        <v>54</v>
+      </c>
+      <c r="C11" t="s">
+        <v>57</v>
+      </c>
       <c r="D11" t="s">
-        <v>46</v>
+        <v>60</v>
+      </c>
+      <c r="E11" t="s">
+        <v>50</v>
+      </c>
+      <c r="F11" t="s">
+        <v>60</v>
+      </c>
+      <c r="G11" t="s">
+        <v>50</v>
       </c>
     </row>
-    <row r="12" ht="15" customHeight="1" spans="4:4" x14ac:dyDescent="0.25"/>
-    <row r="13" ht="15" customHeight="1" x14ac:dyDescent="0.25"/>
-    <row r="14" ht="15" customHeight="1" x14ac:dyDescent="0.25"/>
+    <row r="12" ht="15" customHeight="1" spans="1:7" x14ac:dyDescent="0.25">
+      <c r="A12" t="s">
+        <v>57</v>
+      </c>
+      <c r="B12" t="s">
+        <v>58</v>
+      </c>
+      <c r="C12" t="s">
+        <v>50</v>
+      </c>
+      <c r="D12" t="s">
+        <v>50</v>
+      </c>
+    </row>
+    <row r="13" ht="15" customHeight="1" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="A13" t="s">
+        <v>50</v>
+      </c>
+      <c r="B13" t="s">
+        <v>50</v>
+      </c>
+    </row>
+    <row r="14" ht="15" customHeight="1" spans="1:2" x14ac:dyDescent="0.25"/>
     <row r="15" ht="15" customHeight="1" x14ac:dyDescent="0.25"/>
     <row r="16" ht="15" customHeight="1" x14ac:dyDescent="0.25"/>
     <row r="17" ht="15" customHeight="1" x14ac:dyDescent="0.25"/>
@@ -1605,7 +1965,7 @@
 
 <file path=xl/worksheets/sheet3.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" mc:Ignorable="x14ac">
-  <dimension ref="A3:I42"/>
+  <dimension ref="A3:O42"/>
   <sheetFormatPr defaultRowHeight="14.45" outlineLevelRow="0" outlineLevelCol="0" x14ac:dyDescent="0.25" customHeight="1"/>
   <cols>
     <col min="1" max="1" width="17.85546875" customWidth="1"/>
@@ -1638,41 +1998,59 @@
     <col min="98" max="98" width="19.7109375" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="3" ht="15" customHeight="1" spans="1:9" x14ac:dyDescent="0.25">
+    <row r="3" ht="15" customHeight="1" spans="1:15" x14ac:dyDescent="0.25">
       <c r="A3" t="s">
+        <v>45</v>
+      </c>
+      <c r="B3" t="s">
         <v>46</v>
       </c>
-      <c r="B3" t="s">
+      <c r="C3" t="s">
         <v>47</v>
       </c>
-      <c r="C3" t="s">
+      <c r="D3" t="s">
+        <v>55</v>
+      </c>
+      <c r="E3" t="s">
         <v>49</v>
       </c>
-      <c r="D3" t="s">
-        <v>54</v>
-      </c>
-      <c r="E3" t="s">
-        <v>50</v>
-      </c>
       <c r="F3" t="s">
-        <v>51</v>
+        <v>53</v>
       </c>
       <c r="G3" t="s">
         <v>52</v>
       </c>
       <c r="H3" t="s">
-        <v>53</v>
+        <v>51</v>
       </c>
       <c r="I3" t="s">
-        <v>55</v>
+        <v>56</v>
+      </c>
+      <c r="J3" t="s">
+        <v>54</v>
+      </c>
+      <c r="K3" t="s">
+        <v>59</v>
+      </c>
+      <c r="L3" t="s">
+        <v>58</v>
+      </c>
+      <c r="M3" t="s">
+        <v>57</v>
+      </c>
+      <c r="N3" t="s">
+        <v>60</v>
+      </c>
+      <c r="O3" t="s">
+        <v>50</v>
       </c>
     </row>
-    <row r="4" ht="15" customHeight="1" spans="1:9" x14ac:dyDescent="0.25">
+    <row r="4" ht="15" customHeight="1" spans="1:15" x14ac:dyDescent="0.25">
       <c r="A4" t="s">
-        <v>14</v>
+        <v>12</v>
       </c>
       <c r="B4" t="s">
-        <v>18</v>
+        <v>21</v>
       </c>
       <c r="C4" t="s">
         <v>6</v>
@@ -1681,56 +2059,92 @@
         <v>6</v>
       </c>
       <c r="E4" t="s">
-        <v>44</v>
+        <v>40</v>
       </c>
       <c r="F4" t="s">
-        <v>28</v>
+        <v>25</v>
       </c>
       <c r="G4" t="s">
-        <v>26</v>
+        <v>16</v>
       </c>
       <c r="H4" t="s">
+        <v>32</v>
+      </c>
+      <c r="I4" t="s">
+        <v>1</v>
+      </c>
+      <c r="J4" t="s">
+        <v>27</v>
+      </c>
+      <c r="K4" t="s">
+        <v>6</v>
+      </c>
+      <c r="L4" t="s">
+        <v>16</v>
+      </c>
+      <c r="M4" t="s">
+        <v>27</v>
+      </c>
+      <c r="N4" t="s">
+        <v>15</v>
+      </c>
+      <c r="O4" t="s">
+        <v>27</v>
+      </c>
+    </row>
+    <row r="5" ht="15" customHeight="1" spans="1:15" x14ac:dyDescent="0.25">
+      <c r="A5" t="s">
+        <v>2</v>
+      </c>
+      <c r="B5" t="s">
+        <v>33</v>
+      </c>
+      <c r="C5" t="s">
+        <v>10</v>
+      </c>
+      <c r="D5" t="s">
+        <v>10</v>
+      </c>
+      <c r="E5" t="s">
+        <v>9</v>
+      </c>
+      <c r="F5" t="s">
         <v>22</v>
       </c>
-      <c r="I4" t="s">
+      <c r="G5" t="s">
         <v>3</v>
       </c>
+      <c r="H5" t="s">
+        <v>30</v>
+      </c>
+      <c r="I5" t="s">
+        <v>18</v>
+      </c>
+      <c r="J5" t="s">
+        <v>15</v>
+      </c>
+      <c r="K5" t="s">
+        <v>2</v>
+      </c>
+      <c r="L5" t="s">
+        <v>1</v>
+      </c>
+      <c r="M5" t="s">
+        <v>12</v>
+      </c>
+      <c r="N5" t="s">
+        <v>10</v>
+      </c>
+      <c r="O5" t="s">
+        <v>2</v>
+      </c>
     </row>
-    <row r="5" ht="15" customHeight="1" spans="1:9" x14ac:dyDescent="0.25">
-      <c r="A5" t="s">
-        <v>1</v>
-      </c>
-      <c r="B5" t="s">
-        <v>24</v>
-      </c>
-      <c r="C5" t="s">
+    <row r="6" ht="15" customHeight="1" spans="1:15" x14ac:dyDescent="0.25">
+      <c r="A6" t="s">
         <v>8</v>
       </c>
-      <c r="D5" t="s">
-        <v>8</v>
-      </c>
-      <c r="E5" t="s">
-        <v>7</v>
-      </c>
-      <c r="F5" t="s">
+      <c r="B6" t="s">
         <v>23</v>
-      </c>
-      <c r="G5" t="s">
-        <v>2</v>
-      </c>
-      <c r="H5" t="s">
-        <v>16</v>
-      </c>
-      <c r="I5" t="s">
-        <v>40</v>
-      </c>
-    </row>
-    <row r="6" ht="15" customHeight="1" spans="1:9" x14ac:dyDescent="0.25">
-      <c r="A6" t="s">
-        <v>15</v>
-      </c>
-      <c r="B6" t="s">
-        <v>25</v>
       </c>
       <c r="C6" t="s">
         <v>4</v>
@@ -1739,27 +2153,45 @@
         <v>4</v>
       </c>
       <c r="E6" t="s">
-        <v>36</v>
+        <v>28</v>
       </c>
       <c r="F6" t="s">
-        <v>20</v>
+        <v>14</v>
       </c>
       <c r="G6" t="s">
-        <v>37</v>
+        <v>41</v>
       </c>
       <c r="H6" t="s">
-        <v>9</v>
+        <v>19</v>
       </c>
       <c r="I6" t="s">
-        <v>9</v>
+        <v>19</v>
+      </c>
+      <c r="J6" t="s">
+        <v>38</v>
+      </c>
+      <c r="K6" t="s">
+        <v>14</v>
+      </c>
+      <c r="L6" t="s">
+        <v>23</v>
+      </c>
+      <c r="M6" t="s">
+        <v>4</v>
+      </c>
+      <c r="N6" t="s">
+        <v>11</v>
+      </c>
+      <c r="O6" t="s">
+        <v>17</v>
       </c>
     </row>
-    <row r="7" ht="15" customHeight="1" spans="1:9" x14ac:dyDescent="0.25">
+    <row r="7" ht="15" customHeight="1" spans="1:15" x14ac:dyDescent="0.25">
       <c r="A7" t="s">
-        <v>31</v>
+        <v>34</v>
       </c>
       <c r="B7" t="s">
-        <v>37</v>
+        <v>41</v>
       </c>
       <c r="C7" t="s">
         <v>5</v>
@@ -1768,145 +2200,247 @@
         <v>5</v>
       </c>
       <c r="E7" t="s">
-        <v>43</v>
+        <v>39</v>
       </c>
       <c r="F7" t="s">
+        <v>7</v>
+      </c>
+      <c r="G7" t="s">
+        <v>24</v>
+      </c>
+      <c r="H7" t="s">
         <v>11</v>
       </c>
-      <c r="G7" t="s">
-        <v>27</v>
-      </c>
-      <c r="H7" t="s">
-        <v>10</v>
-      </c>
       <c r="I7" t="s">
+        <v>17</v>
+      </c>
+      <c r="J7" t="s">
+        <v>42</v>
+      </c>
+      <c r="K7" t="s">
+        <v>8</v>
+      </c>
+      <c r="L7" t="s">
+        <v>41</v>
+      </c>
+      <c r="M7" t="s">
+        <v>35</v>
+      </c>
+      <c r="N7" t="s">
+        <v>13</v>
+      </c>
+      <c r="O7" t="s">
+        <v>8</v>
+      </c>
+    </row>
+    <row r="8" ht="15" customHeight="1" spans="1:15" x14ac:dyDescent="0.25">
+      <c r="A8" t="s">
+        <v>30</v>
+      </c>
+      <c r="B8" t="s">
+        <v>22</v>
+      </c>
+      <c r="C8" t="s">
+        <v>12</v>
+      </c>
+      <c r="E8" t="s">
+        <v>12</v>
+      </c>
+      <c r="F8" t="s">
+        <v>2</v>
+      </c>
+      <c r="G8" t="s">
+        <v>1</v>
+      </c>
+      <c r="H8" t="s">
+        <v>9</v>
+      </c>
+      <c r="J8" t="s">
+        <v>3</v>
+      </c>
+      <c r="K8" t="s">
+        <v>16</v>
+      </c>
+      <c r="L8" t="s">
         <v>29</v>
       </c>
+      <c r="M8" t="s">
+        <v>6</v>
+      </c>
+      <c r="N8" t="s">
+        <v>3</v>
+      </c>
+      <c r="O8" t="s">
+        <v>3</v>
+      </c>
     </row>
-    <row r="8" ht="15" customHeight="1" spans="1:9" x14ac:dyDescent="0.25">
-      <c r="A8" t="s">
-        <v>16</v>
-      </c>
-      <c r="B8" t="s">
-        <v>23</v>
-      </c>
-      <c r="C8" t="s">
-        <v>14</v>
-      </c>
-      <c r="E8" t="s">
-        <v>14</v>
-      </c>
-      <c r="F8" t="s">
-        <v>1</v>
-      </c>
-      <c r="G8" t="s">
-        <v>3</v>
-      </c>
-      <c r="H8" t="s">
-        <v>7</v>
-      </c>
-    </row>
-    <row r="9" ht="15" customHeight="1" spans="1:8" x14ac:dyDescent="0.25">
+    <row r="9" ht="15" customHeight="1" spans="1:15" x14ac:dyDescent="0.25">
       <c r="A9" t="s">
         <v>0</v>
       </c>
       <c r="B9" t="s">
-        <v>12</v>
+        <v>29</v>
       </c>
       <c r="C9" t="s">
-        <v>21</v>
+        <v>15</v>
       </c>
       <c r="E9" t="s">
         <v>0</v>
       </c>
       <c r="F9" t="s">
-        <v>16</v>
+        <v>30</v>
       </c>
       <c r="G9" t="s">
         <v>0</v>
       </c>
       <c r="H9" t="s">
-        <v>1</v>
+        <v>2</v>
+      </c>
+      <c r="J9" t="s">
+        <v>30</v>
+      </c>
+      <c r="K9" t="s">
+        <v>21</v>
+      </c>
+      <c r="L9" t="s">
+        <v>9</v>
+      </c>
+      <c r="M9" t="s">
+        <v>0</v>
+      </c>
+      <c r="N9" t="s">
+        <v>9</v>
+      </c>
+      <c r="O9" t="s">
+        <v>9</v>
       </c>
     </row>
-    <row r="10" ht="15" customHeight="1" spans="1:8" x14ac:dyDescent="0.25">
+    <row r="10" ht="15" customHeight="1" spans="1:15" x14ac:dyDescent="0.25">
       <c r="A10" t="s">
-        <v>32</v>
+        <v>35</v>
       </c>
       <c r="B10" t="s">
         <v>4</v>
       </c>
       <c r="C10" t="s">
-        <v>15</v>
+        <v>8</v>
       </c>
       <c r="E10" t="s">
-        <v>10</v>
+        <v>11</v>
       </c>
       <c r="F10" t="s">
-        <v>10</v>
+        <v>11</v>
       </c>
       <c r="G10" t="s">
         <v>4</v>
       </c>
       <c r="H10" t="s">
-        <v>35</v>
+        <v>43</v>
+      </c>
+      <c r="J10" t="s">
+        <v>17</v>
+      </c>
+      <c r="K10" t="s">
+        <v>31</v>
+      </c>
+      <c r="L10" t="s">
+        <v>38</v>
+      </c>
+      <c r="M10" t="s">
+        <v>8</v>
+      </c>
+      <c r="N10" t="s">
+        <v>5</v>
+      </c>
+      <c r="O10" t="s">
+        <v>34</v>
       </c>
     </row>
-    <row r="11" ht="15" customHeight="1" spans="1:8" x14ac:dyDescent="0.25">
+    <row r="11" ht="15" customHeight="1" spans="1:15" x14ac:dyDescent="0.25">
       <c r="A11" t="s">
-        <v>17</v>
+        <v>13</v>
       </c>
       <c r="B11" t="s">
         <v>5</v>
       </c>
       <c r="C11" t="s">
-        <v>17</v>
+        <v>13</v>
       </c>
       <c r="E11" t="s">
-        <v>15</v>
+        <v>8</v>
       </c>
       <c r="F11" t="s">
-        <v>30</v>
+        <v>26</v>
       </c>
       <c r="G11" t="s">
         <v>5</v>
       </c>
       <c r="H11" t="s">
-        <v>30</v>
+        <v>26</v>
+      </c>
+      <c r="J11" t="s">
+        <v>8</v>
+      </c>
+      <c r="K11" t="s">
+        <v>23</v>
+      </c>
+      <c r="L11" t="s">
+        <v>13</v>
+      </c>
+      <c r="M11" t="s">
+        <v>5</v>
+      </c>
+      <c r="N11" t="s">
+        <v>7</v>
+      </c>
+      <c r="O11" t="s">
+        <v>7</v>
       </c>
     </row>
-    <row r="12" ht="15" customHeight="1" spans="1:8" x14ac:dyDescent="0.25">
+    <row r="12" ht="15" customHeight="1" spans="1:15" x14ac:dyDescent="0.25">
       <c r="A12" t="s">
-        <v>18</v>
+        <v>21</v>
       </c>
       <c r="B12" t="s">
+        <v>3</v>
+      </c>
+      <c r="C12" t="s">
+        <v>3</v>
+      </c>
+      <c r="E12" t="s">
+        <v>33</v>
+      </c>
+      <c r="F12" t="s">
+        <v>27</v>
+      </c>
+      <c r="H12" t="s">
+        <v>1</v>
+      </c>
+      <c r="J12" t="s">
+        <v>40</v>
+      </c>
+      <c r="L12" t="s">
+        <v>25</v>
+      </c>
+      <c r="M12" t="s">
         <v>2</v>
       </c>
-      <c r="C12" t="s">
-        <v>2</v>
-      </c>
-      <c r="E12" t="s">
-        <v>24</v>
-      </c>
-      <c r="F12" t="s">
-        <v>34</v>
-      </c>
-      <c r="H12" t="s">
-        <v>3</v>
+      <c r="O12" t="s">
+        <v>40</v>
       </c>
     </row>
-    <row r="13" ht="15" customHeight="1" spans="1:8" x14ac:dyDescent="0.25">
+    <row r="13" ht="15" customHeight="1" spans="1:15" x14ac:dyDescent="0.25">
       <c r="A13" t="s">
-        <v>3</v>
+        <v>1</v>
       </c>
       <c r="B13" t="s">
         <v>0</v>
       </c>
       <c r="C13" t="s">
-        <v>40</v>
+        <v>18</v>
       </c>
       <c r="E13" t="s">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="F13" t="s">
         <v>6</v>
@@ -1914,240 +2448,372 @@
       <c r="H13" t="s">
         <v>0</v>
       </c>
+      <c r="J13" t="s">
+        <v>1</v>
+      </c>
+      <c r="L13" t="s">
+        <v>12</v>
+      </c>
+      <c r="M13" t="s">
+        <v>18</v>
+      </c>
+      <c r="O13" t="s">
+        <v>1</v>
+      </c>
     </row>
-    <row r="14" ht="15" customHeight="1" spans="1:8" x14ac:dyDescent="0.25">
+    <row r="14" ht="15" customHeight="1" spans="1:15" x14ac:dyDescent="0.25">
       <c r="A14" t="s">
+        <v>31</v>
+      </c>
+      <c r="B14" t="s">
+        <v>11</v>
+      </c>
+      <c r="C14" t="s">
         <v>19</v>
       </c>
-      <c r="B14" t="s">
-        <v>10</v>
-      </c>
-      <c r="C14" t="s">
-        <v>9</v>
-      </c>
       <c r="E14" t="s">
+        <v>38</v>
+      </c>
+      <c r="F14" t="s">
+        <v>31</v>
+      </c>
+      <c r="H14" t="s">
+        <v>31</v>
+      </c>
+      <c r="J14" t="s">
         <v>39</v>
       </c>
-      <c r="F14" t="s">
-        <v>19</v>
-      </c>
-      <c r="H14" t="s">
-        <v>19</v>
+      <c r="L14" t="s">
+        <v>4</v>
+      </c>
+      <c r="M14" t="s">
+        <v>14</v>
+      </c>
+      <c r="O14" t="s">
+        <v>36</v>
       </c>
     </row>
-    <row r="15" ht="15" customHeight="1" spans="1:8" x14ac:dyDescent="0.25">
+    <row r="15" ht="15" customHeight="1" spans="1:15" x14ac:dyDescent="0.25">
       <c r="A15" t="s">
-        <v>33</v>
+        <v>36</v>
       </c>
       <c r="B15" t="s">
-        <v>11</v>
+        <v>7</v>
       </c>
       <c r="C15" t="s">
-        <v>41</v>
+        <v>42</v>
       </c>
       <c r="E15" t="s">
-        <v>17</v>
+        <v>13</v>
       </c>
       <c r="F15" t="s">
-        <v>41</v>
+        <v>42</v>
       </c>
       <c r="H15" t="s">
+        <v>24</v>
+      </c>
+      <c r="J15" t="s">
+        <v>26</v>
+      </c>
+      <c r="L15" t="s">
+        <v>5</v>
+      </c>
+      <c r="M15" t="s">
+        <v>20</v>
+      </c>
+      <c r="O15" t="s">
+        <v>37</v>
+      </c>
+    </row>
+    <row r="16" ht="15" customHeight="1" spans="1:15" x14ac:dyDescent="0.25">
+      <c r="A16" t="s">
         <v>27</v>
       </c>
-    </row>
-    <row r="16" ht="15" customHeight="1" spans="1:8" x14ac:dyDescent="0.25">
-      <c r="A16" t="s">
-        <v>34</v>
-      </c>
       <c r="B16" t="s">
-        <v>26</v>
+        <v>16</v>
       </c>
       <c r="C16" t="s">
-        <v>26</v>
+        <v>16</v>
       </c>
       <c r="E16" t="s">
-        <v>28</v>
+        <v>25</v>
       </c>
       <c r="F16" t="s">
-        <v>21</v>
+        <v>15</v>
       </c>
       <c r="H16" t="s">
         <v>6</v>
       </c>
+      <c r="J16" t="s">
+        <v>32</v>
+      </c>
+      <c r="L16" t="s">
+        <v>15</v>
+      </c>
+      <c r="M16" t="s">
+        <v>22</v>
+      </c>
+      <c r="O16" t="s">
+        <v>25</v>
+      </c>
     </row>
-    <row r="17" ht="15" customHeight="1" spans="1:8" x14ac:dyDescent="0.25">
+    <row r="17" ht="15" customHeight="1" spans="1:15" x14ac:dyDescent="0.25">
       <c r="A17" t="s">
-        <v>8</v>
+        <v>10</v>
       </c>
       <c r="B17" t="s">
+        <v>1</v>
+      </c>
+      <c r="C17" t="s">
+        <v>2</v>
+      </c>
+      <c r="E17" t="s">
+        <v>29</v>
+      </c>
+      <c r="F17" t="s">
         <v>3</v>
       </c>
-      <c r="C17" t="s">
+      <c r="H17" t="s">
+        <v>29</v>
+      </c>
+      <c r="J17" t="s">
+        <v>0</v>
+      </c>
+      <c r="L17" t="s">
+        <v>21</v>
+      </c>
+      <c r="M17" t="s">
+        <v>33</v>
+      </c>
+      <c r="O17" t="s">
+        <v>12</v>
+      </c>
+    </row>
+    <row r="18" ht="15" customHeight="1" spans="1:15" x14ac:dyDescent="0.25">
+      <c r="A18" t="s">
+        <v>19</v>
+      </c>
+      <c r="B18" t="s">
+        <v>37</v>
+      </c>
+      <c r="C18" t="s">
+        <v>23</v>
+      </c>
+      <c r="E18" t="s">
+        <v>14</v>
+      </c>
+      <c r="F18" t="s">
+        <v>28</v>
+      </c>
+      <c r="H18" t="s">
+        <v>17</v>
+      </c>
+      <c r="J18" t="s">
+        <v>34</v>
+      </c>
+      <c r="L18" t="s">
+        <v>28</v>
+      </c>
+      <c r="M18" t="s">
+        <v>28</v>
+      </c>
+      <c r="O18" t="s">
+        <v>35</v>
+      </c>
+    </row>
+    <row r="19" ht="15" customHeight="1" spans="1:15" x14ac:dyDescent="0.25">
+      <c r="A19" t="s">
+        <v>14</v>
+      </c>
+      <c r="B19" t="s">
+        <v>24</v>
+      </c>
+      <c r="C19" t="s">
+        <v>20</v>
+      </c>
+      <c r="E19" t="s">
+        <v>35</v>
+      </c>
+      <c r="F19" t="s">
+        <v>23</v>
+      </c>
+      <c r="H19" t="s">
+        <v>20</v>
+      </c>
+      <c r="J19" t="s">
+        <v>7</v>
+      </c>
+      <c r="L19" t="s">
+        <v>37</v>
+      </c>
+      <c r="M19" t="s">
+        <v>36</v>
+      </c>
+      <c r="O19" t="s">
+        <v>44</v>
+      </c>
+    </row>
+    <row r="20" ht="15" customHeight="1" spans="1:15" x14ac:dyDescent="0.25">
+      <c r="A20" t="s">
+        <v>15</v>
+      </c>
+      <c r="B20" t="s">
+        <v>25</v>
+      </c>
+      <c r="C20" t="s">
         <v>1</v>
       </c>
-      <c r="E17" t="s">
-        <v>12</v>
-      </c>
-      <c r="F17" t="s">
+      <c r="E20" t="s">
+        <v>32</v>
+      </c>
+      <c r="F20" t="s">
+        <v>21</v>
+      </c>
+      <c r="J20" t="s">
+        <v>18</v>
+      </c>
+      <c r="L20" t="s">
+        <v>22</v>
+      </c>
+      <c r="O20" t="s">
+        <v>16</v>
+      </c>
+    </row>
+    <row r="21" ht="15" customHeight="1" spans="1:15" x14ac:dyDescent="0.25">
+      <c r="A21" t="s">
+        <v>32</v>
+      </c>
+      <c r="B21" t="s">
         <v>2</v>
-      </c>
-      <c r="H17" t="s">
-        <v>12</v>
-      </c>
-    </row>
-    <row r="18" ht="15" customHeight="1" spans="1:8" x14ac:dyDescent="0.25">
-      <c r="A18" t="s">
-        <v>9</v>
-      </c>
-      <c r="B18" t="s">
-        <v>38</v>
-      </c>
-      <c r="C18" t="s">
-        <v>25</v>
-      </c>
-      <c r="E18" t="s">
-        <v>20</v>
-      </c>
-      <c r="F18" t="s">
-        <v>36</v>
-      </c>
-      <c r="H18" t="s">
-        <v>29</v>
-      </c>
-    </row>
-    <row r="19" ht="15" customHeight="1" spans="1:8" x14ac:dyDescent="0.25">
-      <c r="A19" t="s">
-        <v>20</v>
-      </c>
-      <c r="B19" t="s">
-        <v>27</v>
-      </c>
-      <c r="C19" t="s">
-        <v>13</v>
-      </c>
-      <c r="E19" t="s">
-        <v>32</v>
-      </c>
-      <c r="F19" t="s">
-        <v>25</v>
-      </c>
-      <c r="H19" t="s">
-        <v>13</v>
-      </c>
-    </row>
-    <row r="20" ht="15" customHeight="1" spans="1:8" x14ac:dyDescent="0.25">
-      <c r="A20" t="s">
-        <v>21</v>
-      </c>
-      <c r="B20" t="s">
-        <v>28</v>
-      </c>
-      <c r="C20" t="s">
-        <v>3</v>
-      </c>
-      <c r="E20" t="s">
-        <v>22</v>
-      </c>
-      <c r="F20" t="s">
-        <v>18</v>
-      </c>
-    </row>
-    <row r="21" ht="15" customHeight="1" spans="1:6" x14ac:dyDescent="0.25">
-      <c r="A21" t="s">
-        <v>22</v>
-      </c>
-      <c r="B21" t="s">
-        <v>1</v>
       </c>
       <c r="C21" t="s">
         <v>0</v>
       </c>
       <c r="E21" t="s">
-        <v>2</v>
+        <v>3</v>
       </c>
       <c r="F21" t="s">
+        <v>33</v>
+      </c>
+      <c r="J21" t="s">
+        <v>10</v>
+      </c>
+      <c r="L21" t="s">
+        <v>40</v>
+      </c>
+      <c r="O21" t="s">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="22" ht="15" customHeight="1" spans="1:15" x14ac:dyDescent="0.25">
+      <c r="A22" t="s">
+        <v>11</v>
+      </c>
+      <c r="B22" t="s">
+        <v>17</v>
+      </c>
+      <c r="C22" t="s">
+        <v>39</v>
+      </c>
+      <c r="E22" t="s">
+        <v>34</v>
+      </c>
+      <c r="F22" t="s">
+        <v>36</v>
+      </c>
+      <c r="J22" t="s">
         <v>24</v>
       </c>
+      <c r="L22" t="s">
+        <v>39</v>
+      </c>
+      <c r="O22" t="s">
+        <v>4</v>
+      </c>
     </row>
-    <row r="22" ht="15" customHeight="1" spans="1:6" x14ac:dyDescent="0.25">
-      <c r="A22" t="s">
-        <v>10</v>
-      </c>
-      <c r="B22" t="s">
-        <v>29</v>
-      </c>
-      <c r="C22" t="s">
-        <v>43</v>
-      </c>
-      <c r="E22" t="s">
-        <v>31</v>
-      </c>
-      <c r="F22" t="s">
-        <v>33</v>
+    <row r="23" ht="15" customHeight="1" spans="1:15" x14ac:dyDescent="0.25">
+      <c r="A23" t="s">
+        <v>17</v>
+      </c>
+      <c r="B23" t="s">
+        <v>20</v>
+      </c>
+      <c r="C23" t="s">
+        <v>9</v>
+      </c>
+      <c r="E23" t="s">
+        <v>7</v>
+      </c>
+      <c r="F23" t="s">
+        <v>37</v>
+      </c>
+      <c r="J23" t="s">
+        <v>13</v>
+      </c>
+      <c r="L23" t="s">
+        <v>26</v>
+      </c>
+      <c r="O23" t="s">
+        <v>24</v>
       </c>
     </row>
-    <row r="23" ht="15" customHeight="1" spans="1:6" x14ac:dyDescent="0.25">
-      <c r="A23" t="s">
-        <v>29</v>
-      </c>
-      <c r="B23" t="s">
-        <v>13</v>
-      </c>
-      <c r="C23" t="s">
-        <v>7</v>
-      </c>
-      <c r="E23" t="s">
-        <v>11</v>
-      </c>
-      <c r="F23" t="s">
-        <v>38</v>
-      </c>
-    </row>
-    <row r="24" ht="15" customHeight="1" spans="1:6" x14ac:dyDescent="0.25">
+    <row r="24" ht="15" customHeight="1" spans="1:15" x14ac:dyDescent="0.25">
       <c r="A24" t="s">
-        <v>23</v>
+        <v>22</v>
       </c>
       <c r="B24" t="s">
         <v>6</v>
       </c>
       <c r="F24" t="s">
+        <v>1</v>
+      </c>
+      <c r="O24" t="s">
+        <v>6</v>
+      </c>
+    </row>
+    <row r="25" ht="15" customHeight="1" spans="1:15" x14ac:dyDescent="0.25">
+      <c r="A25" t="s">
         <v>3</v>
       </c>
-    </row>
-    <row r="25" ht="15" customHeight="1" spans="1:6" x14ac:dyDescent="0.25">
-      <c r="A25" t="s">
-        <v>2</v>
-      </c>
       <c r="B25" t="s">
-        <v>8</v>
+        <v>10</v>
       </c>
       <c r="F25" t="s">
         <v>0</v>
       </c>
+      <c r="O25" t="s">
+        <v>18</v>
+      </c>
     </row>
-    <row r="26" ht="15" customHeight="1" spans="1:6" x14ac:dyDescent="0.25">
+    <row r="26" ht="15" customHeight="1" spans="1:15" x14ac:dyDescent="0.25">
       <c r="A26" t="s">
-        <v>36</v>
+        <v>28</v>
       </c>
       <c r="B26" t="s">
-        <v>20</v>
+        <v>14</v>
       </c>
       <c r="F26" t="s">
         <v>4</v>
       </c>
+      <c r="O26" t="s">
+        <v>19</v>
+      </c>
     </row>
-    <row r="27" ht="15" customHeight="1" spans="1:6" x14ac:dyDescent="0.25">
+    <row r="27" ht="15" customHeight="1" spans="1:15" x14ac:dyDescent="0.25">
       <c r="A27" t="s">
-        <v>11</v>
+        <v>7</v>
       </c>
       <c r="B27" t="s">
-        <v>39</v>
+        <v>38</v>
       </c>
       <c r="F27" t="s">
         <v>5</v>
       </c>
+      <c r="O27" t="s">
+        <v>20</v>
+      </c>
     </row>
-    <row r="28" ht="15" customHeight="1" spans="1:6" x14ac:dyDescent="0.25"/>
+    <row r="28" ht="15" customHeight="1" spans="6:15" x14ac:dyDescent="0.25"/>
     <row r="29" ht="15" customHeight="1" x14ac:dyDescent="0.25"/>
     <row r="30" ht="15" customHeight="1" x14ac:dyDescent="0.25"/>
     <row r="31" ht="15" customHeight="1" x14ac:dyDescent="0.25"/>
@@ -2169,7 +2835,7 @@
 
 <file path=xl/worksheets/sheet4.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" mc:Ignorable="x14ac">
-  <dimension ref="A3:I1898"/>
+  <dimension ref="A3:O1898"/>
   <sheetFormatPr defaultRowHeight="14.45" outlineLevelRow="0" outlineLevelCol="0" x14ac:dyDescent="0.25" customHeight="1"/>
   <cols>
     <col min="1" max="1" width="55.28515625" customWidth="1"/>
@@ -2253,159 +2919,249 @@
     <col min="99" max="99" width="47.7109375" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="3" ht="15" customHeight="1" spans="1:9" x14ac:dyDescent="0.25">
+    <row r="3" ht="15" customHeight="1" spans="1:15" x14ac:dyDescent="0.25">
       <c r="A3" t="s">
+        <v>45</v>
+      </c>
+      <c r="B3" t="s">
         <v>46</v>
       </c>
-      <c r="B3" t="s">
+      <c r="C3" t="s">
         <v>47</v>
       </c>
-      <c r="C3" t="s">
+      <c r="D3" t="s">
+        <v>55</v>
+      </c>
+      <c r="E3" t="s">
         <v>49</v>
       </c>
-      <c r="D3" t="s">
-        <v>54</v>
-      </c>
-      <c r="E3" t="s">
-        <v>50</v>
-      </c>
       <c r="F3" t="s">
-        <v>51</v>
+        <v>53</v>
       </c>
       <c r="G3" t="s">
         <v>52</v>
       </c>
       <c r="H3" t="s">
-        <v>53</v>
+        <v>51</v>
       </c>
       <c r="I3" t="s">
-        <v>55</v>
+        <v>56</v>
+      </c>
+      <c r="J3" t="s">
+        <v>54</v>
+      </c>
+      <c r="K3" t="s">
+        <v>59</v>
+      </c>
+      <c r="L3" t="s">
+        <v>58</v>
+      </c>
+      <c r="M3" t="s">
+        <v>57</v>
+      </c>
+      <c r="N3" t="s">
+        <v>60</v>
+      </c>
+      <c r="O3" t="s">
+        <v>50</v>
       </c>
     </row>
-    <row r="4" ht="15" customHeight="1" spans="1:9" x14ac:dyDescent="0.25">
+    <row r="4" ht="15" customHeight="1" spans="1:15" x14ac:dyDescent="0.25">
       <c r="A4" t="s">
-        <v>56</v>
+        <v>61</v>
       </c>
       <c r="B4" t="s">
-        <v>57</v>
+        <v>62</v>
       </c>
       <c r="C4" t="s">
-        <v>58</v>
+        <v>63</v>
       </c>
       <c r="D4" t="s">
-        <v>59</v>
+        <v>64</v>
       </c>
       <c r="E4" t="s">
-        <v>60</v>
+        <v>65</v>
       </c>
       <c r="F4" t="s">
-        <v>61</v>
+        <v>66</v>
       </c>
       <c r="G4" t="s">
-        <v>62</v>
+        <v>67</v>
       </c>
       <c r="H4" t="s">
-        <v>63</v>
+        <v>68</v>
       </c>
       <c r="I4" t="s">
-        <v>64</v>
+        <v>69</v>
+      </c>
+      <c r="J4" t="s">
+        <v>70</v>
+      </c>
+      <c r="K4" t="s">
+        <v>71</v>
+      </c>
+      <c r="L4" t="s">
+        <v>72</v>
+      </c>
+      <c r="M4" t="s">
+        <v>73</v>
+      </c>
+      <c r="N4" t="s">
+        <v>74</v>
+      </c>
+      <c r="O4" t="s">
+        <v>75</v>
       </c>
     </row>
-    <row r="5" ht="15" customHeight="1" spans="1:9" x14ac:dyDescent="0.25">
+    <row r="5" ht="15" customHeight="1" spans="1:15" x14ac:dyDescent="0.25">
       <c r="A5" t="s">
-        <v>65</v>
+        <v>76</v>
       </c>
       <c r="B5" t="s">
-        <v>66</v>
+        <v>77</v>
       </c>
       <c r="C5" t="s">
-        <v>67</v>
+        <v>78</v>
       </c>
       <c r="E5" t="s">
-        <v>68</v>
+        <v>79</v>
       </c>
       <c r="F5" t="s">
-        <v>69</v>
+        <v>80</v>
       </c>
       <c r="G5" t="s">
-        <v>70</v>
+        <v>81</v>
       </c>
       <c r="H5" t="s">
-        <v>71</v>
+        <v>82</v>
+      </c>
+      <c r="J5" t="s">
+        <v>83</v>
+      </c>
+      <c r="K5" t="s">
+        <v>84</v>
+      </c>
+      <c r="L5" t="s">
+        <v>85</v>
+      </c>
+      <c r="M5" t="s">
+        <v>86</v>
+      </c>
+      <c r="N5" t="s">
+        <v>87</v>
+      </c>
+      <c r="O5" t="s">
+        <v>88</v>
       </c>
     </row>
-    <row r="6" ht="15" customHeight="1" spans="1:8" x14ac:dyDescent="0.25">
+    <row r="6" ht="15" customHeight="1" spans="1:15" x14ac:dyDescent="0.25">
       <c r="A6" t="s">
-        <v>72</v>
+        <v>89</v>
       </c>
       <c r="B6" t="s">
-        <v>73</v>
+        <v>90</v>
       </c>
       <c r="C6" t="s">
-        <v>74</v>
+        <v>91</v>
       </c>
       <c r="E6" t="s">
-        <v>75</v>
+        <v>92</v>
       </c>
       <c r="F6" t="s">
-        <v>76</v>
+        <v>93</v>
       </c>
       <c r="H6" t="s">
-        <v>77</v>
+        <v>94</v>
+      </c>
+      <c r="J6" t="s">
+        <v>95</v>
+      </c>
+      <c r="L6" t="s">
+        <v>96</v>
+      </c>
+      <c r="M6" t="s">
+        <v>97</v>
+      </c>
+      <c r="O6" t="s">
+        <v>98</v>
       </c>
     </row>
-    <row r="7" ht="15" customHeight="1" spans="1:8" x14ac:dyDescent="0.25">
+    <row r="7" ht="15" customHeight="1" spans="1:15" x14ac:dyDescent="0.25">
       <c r="A7" t="s">
-        <v>78</v>
+        <v>99</v>
       </c>
       <c r="B7" t="s">
-        <v>79</v>
+        <v>100</v>
       </c>
       <c r="C7" t="s">
-        <v>80</v>
+        <v>101</v>
       </c>
       <c r="E7" t="s">
+        <v>102</v>
+      </c>
+      <c r="F7" t="s">
+        <v>103</v>
+      </c>
+      <c r="H7" t="s">
+        <v>104</v>
+      </c>
+      <c r="J7" t="s">
+        <v>105</v>
+      </c>
+      <c r="L7" t="s">
+        <v>106</v>
+      </c>
+      <c r="M7" t="s">
+        <v>107</v>
+      </c>
+      <c r="O7" t="s">
+        <v>108</v>
+      </c>
+    </row>
+    <row r="8" ht="15" customHeight="1" spans="1:15" x14ac:dyDescent="0.25">
+      <c r="A8" t="s">
+        <v>109</v>
+      </c>
+      <c r="B8" t="s">
+        <v>110</v>
+      </c>
+      <c r="C8" t="s">
+        <v>111</v>
+      </c>
+      <c r="E8" t="s">
+        <v>112</v>
+      </c>
+      <c r="F8" t="s">
+        <v>113</v>
+      </c>
+      <c r="J8" t="s">
+        <v>114</v>
+      </c>
+      <c r="L8" t="s">
+        <v>115</v>
+      </c>
+      <c r="O8" t="s">
+        <v>116</v>
+      </c>
+    </row>
+    <row r="9" ht="15" customHeight="1" spans="1:15" x14ac:dyDescent="0.25">
+      <c r="A9" t="s">
+        <v>117</v>
+      </c>
+      <c r="B9" t="s">
+        <v>118</v>
+      </c>
+      <c r="E9" t="s">
+        <v>119</v>
+      </c>
+      <c r="F9" t="s">
         <v>81</v>
       </c>
-      <c r="F7" t="s">
-        <v>82</v>
-      </c>
-      <c r="H7" t="s">
-        <v>83</v>
+      <c r="O9" t="s">
+        <v>120</v>
       </c>
     </row>
-    <row r="8" ht="15" customHeight="1" spans="1:8" x14ac:dyDescent="0.25">
-      <c r="A8" t="s">
-        <v>84</v>
-      </c>
-      <c r="B8" t="s">
-        <v>85</v>
-      </c>
-      <c r="C8" t="s">
-        <v>86</v>
-      </c>
-      <c r="E8" t="s">
-        <v>87</v>
-      </c>
-      <c r="F8" t="s">
-        <v>88</v>
-      </c>
-    </row>
-    <row r="9" ht="15" customHeight="1" spans="1:6" x14ac:dyDescent="0.25">
-      <c r="A9" t="s">
-        <v>89</v>
-      </c>
-      <c r="B9" t="s">
-        <v>90</v>
-      </c>
-      <c r="E9" t="s">
-        <v>91</v>
-      </c>
-      <c r="F9" t="s">
-        <v>70</v>
-      </c>
-    </row>
-    <row r="10" ht="15" customHeight="1" spans="1:6" x14ac:dyDescent="0.25"/>
+    <row r="10" ht="15" customHeight="1" spans="5:15" x14ac:dyDescent="0.25"/>
     <row r="11" ht="15" customHeight="1" x14ac:dyDescent="0.25"/>
     <row r="12" ht="15" customHeight="1" x14ac:dyDescent="0.25"/>
     <row r="13" ht="15" customHeight="1" x14ac:dyDescent="0.25"/>

</xml_diff>